<commit_message>
Record LT2-1 trunk VLAN change as done
The 22 new VLANs are now tagged on LT2-1 1/1/23 and 1/1/24 (trunks to
LT2-2 and LT2-3), confirmed with show vlan ethernet 1/1/23. Updated the
Switches and Ports without device tabs to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZ7jJsE6GWKm6ehHY39VNr
</commit_message>
<xml_diff>
--- a/200V Device Port List.xlsx
+++ b/200V Device Port List.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5247" uniqueCount="1029">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5247" uniqueCount="1028">
   <si>
     <t xml:space="preserve">Master row</t>
   </si>
@@ -2363,7 +2363,7 @@
     <t xml:space="preserve">10_F0_68_0C_06_D6</t>
   </si>
   <si>
-    <t xml:space="preserve">Via LT2-1 port 1/1/23 (their 1/1/12), confirmed by LLDP</t>
+    <t xml:space="preserve">Via LT2-1 port 1/1/23 (their 1/1/12), confirmed by LLDP. New VLANs tagged on LT2-1 1/1/23 on 6 Oct 2026</t>
   </si>
   <si>
     <t xml:space="preserve">switch-200V-LT2-3</t>
@@ -2372,7 +2372,7 @@
     <t xml:space="preserve">10_F0_68_0B_D2_3E</t>
   </si>
   <si>
-    <t xml:space="preserve">Via LT2-1 port 1/1/24 (their 1/1/12), confirmed by LLDP</t>
+    <t xml:space="preserve">Via LT2-1 port 1/1/24 (their 1/1/12), confirmed by LLDP. New VLANs tagged on LT2-1 1/1/24 on 6 Oct 2026</t>
   </si>
   <si>
     <t xml:space="preserve">switch-200V-8</t>
@@ -2435,25 +2435,22 @@
     <t xml:space="preserve">LLDP: CLA-TAN3130059J (NUC, MAC 48:21:0B:56:AC:A4), not in device list</t>
   </si>
   <si>
-    <t xml:space="preserve">100,1212,1213,1230,1240,1250,1271,1272,1273</t>
+    <t xml:space="preserve">100,1212,1213,1230,1240,1250,1271,1272,1273,2000,2010,2020,2100,2200,2300,2310,2320,2400,2500,2510,2520,2530,2600,2700,2800,2810,2900,2950,2951,2952,2953</t>
   </si>
   <si>
     <t xml:space="preserve">10:F0:68:0C:06:E1, 10:F0:68:0C:06:D6</t>
   </si>
   <si>
-    <t xml:space="preserve">Uplink to switch-200V-LT2-2 (LLDP)</t>
+    <t xml:space="preserve">Uplink to switch-200V-LT2-2 (LLDP). 22 new VLANs (2000-2953) tagged 6 Oct 2026, ahead of cutover</t>
   </si>
   <si>
     <t xml:space="preserve">10:F0:68:0B:D2:49, 10:F0:68:0B:D2:3E, AC:B4:80:F1:61:7F</t>
   </si>
   <si>
-    <t xml:space="preserve">Uplink to switch-200V-LT2-3 (LLDP)</t>
+    <t xml:space="preserve">Uplink to switch-200V-LT2-3 (LLDP). 22 new VLANs (2000-2953) tagged 6 Oct 2026, ahead of cutover</t>
   </si>
   <si>
     <t xml:space="preserve">1212,1213,1230,1250,1271,1272,1273,2000,2010,2020,2100,2200,2300,2310,2320,2400,2500,2510,2520,2530,2600,2700,2800,2810,2900,2950,2951,2952,2953</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100,1212,1213,1230,1240,1250,1271,1272,1273,2000,2010,2020,2100,2200,2300,2310,2320,2400,2500,2510,2520,2530,2600,2700,2800,2810,2900,2950,2951,2952,2953</t>
   </si>
   <si>
     <t xml:space="preserve">1240 (200v_staff)</t>
@@ -17241,7 +17238,7 @@
         <v>794</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>807</v>
+        <v>801</v>
       </c>
       <c r="F33" s="6" t="n">
         <v>0</v>
@@ -17259,13 +17256,13 @@
         <v>14</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>792</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F34" s="2" t="n">
         <v>0</v>
@@ -17281,13 +17278,13 @@
         <v>71</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>792</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F35" s="2" t="n">
         <v>0</v>
@@ -17303,13 +17300,13 @@
         <v>85</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>792</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F36" s="2" t="n">
         <v>0</v>
@@ -17325,19 +17322,19 @@
         <v>22</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D37" s="7" t="s">
         <v>792</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F37" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="H37" s="7"/>
     </row>
@@ -17349,13 +17346,13 @@
         <v>27</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>792</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F38" s="2" t="n">
         <v>0</v>
@@ -17371,13 +17368,13 @@
         <v>31</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>792</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F39" s="2" t="n">
         <v>0</v>
@@ -17393,13 +17390,13 @@
         <v>35</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>792</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F40" s="2" t="n">
         <v>0</v>
@@ -17415,13 +17412,13 @@
         <v>38</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>792</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F41" s="2" t="n">
         <v>0</v>
@@ -17437,13 +17434,13 @@
         <v>99</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>792</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F42" s="2" t="n">
         <v>0</v>
@@ -17459,13 +17456,13 @@
         <v>41</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>792</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F43" s="2" t="n">
         <v>0</v>
@@ -17481,13 +17478,13 @@
         <v>44</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>792</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F44" s="2" t="n">
         <v>0</v>
@@ -17509,7 +17506,7 @@
         <v>794</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>807</v>
+        <v>801</v>
       </c>
       <c r="F45" s="6" t="n">
         <v>0</v>
@@ -17533,7 +17530,7 @@
         <v>794</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="F46" s="6" t="n">
         <v>0</v>
@@ -17551,19 +17548,19 @@
         <v>85</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="D47" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F47" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G47" s="7" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="H47" s="7"/>
     </row>
@@ -17575,22 +17572,22 @@
         <v>99</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="D48" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F48" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G48" s="7" t="s">
+        <v>813</v>
+      </c>
+      <c r="H48" s="7" t="s">
         <v>814</v>
-      </c>
-      <c r="H48" s="7" t="s">
-        <v>815</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17607,7 +17604,7 @@
         <v>794</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F49" s="6" t="n">
         <v>0</v>
@@ -17625,7 +17622,7 @@
         <v>44</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>16</v>
@@ -17651,7 +17648,7 @@
         <v>794</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F51" s="6" t="n">
         <v>0</v>
@@ -17688,7 +17685,7 @@
         <v>80</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>23</v>
@@ -17708,7 +17705,7 @@
         <v>80</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="C54" s="7" t="s">
         <v>15</v>
@@ -17721,7 +17718,7 @@
         <v>1</v>
       </c>
       <c r="G54" s="7" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="H54" s="7"/>
     </row>
@@ -17763,7 +17760,7 @@
         <v>1</v>
       </c>
       <c r="G56" s="7" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="H56" s="7"/>
     </row>
@@ -17845,7 +17842,7 @@
         <v>1</v>
       </c>
       <c r="G60" s="7" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="H60" s="7"/>
     </row>
@@ -17874,7 +17871,7 @@
         <v>80</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>219</v>
@@ -17894,7 +17891,7 @@
         <v>80</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="C63" s="7" t="s">
         <v>219</v>
@@ -17907,7 +17904,7 @@
         <v>1</v>
       </c>
       <c r="G63" s="7" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="H63" s="7"/>
     </row>
@@ -17916,7 +17913,7 @@
         <v>80</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>219</v>
@@ -17936,7 +17933,7 @@
         <v>80</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>219</v>
@@ -18099,10 +18096,10 @@
         <v>590</v>
       </c>
       <c r="C73" s="2" t="s">
+        <v>825</v>
+      </c>
+      <c r="D73" s="2" t="s">
         <v>826</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>827</v>
       </c>
       <c r="E73" s="2"/>
       <c r="F73" s="2" t="n">
@@ -18119,17 +18116,17 @@
         <v>592</v>
       </c>
       <c r="C74" s="7" t="s">
+        <v>825</v>
+      </c>
+      <c r="D74" s="7" t="s">
         <v>826</v>
-      </c>
-      <c r="D74" s="7" t="s">
-        <v>827</v>
       </c>
       <c r="E74" s="7"/>
       <c r="F74" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G74" s="7" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="H74" s="7"/>
     </row>
@@ -18151,7 +18148,7 @@
         <v>1</v>
       </c>
       <c r="G75" s="7" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="H75" s="7"/>
     </row>
@@ -18173,7 +18170,7 @@
         <v>1</v>
       </c>
       <c r="G76" s="7" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="H76" s="7"/>
     </row>
@@ -18195,7 +18192,7 @@
         <v>1</v>
       </c>
       <c r="G77" s="7" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="H77" s="7"/>
     </row>
@@ -18210,7 +18207,7 @@
         <v>792</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E78" s="4"/>
       <c r="F78" s="4" t="n">
@@ -18218,7 +18215,7 @@
       </c>
       <c r="G78" s="4"/>
       <c r="H78" s="4" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18232,7 +18229,7 @@
         <v>792</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E79" s="4"/>
       <c r="F79" s="4" t="n">
@@ -18240,7 +18237,7 @@
       </c>
       <c r="G79" s="4"/>
       <c r="H79" s="4" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18254,7 +18251,7 @@
         <v>792</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E80" s="4"/>
       <c r="F80" s="4" t="n">
@@ -18262,7 +18259,7 @@
       </c>
       <c r="G80" s="4"/>
       <c r="H80" s="4" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18276,7 +18273,7 @@
         <v>792</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E81" s="4"/>
       <c r="F81" s="4" t="n">
@@ -18284,7 +18281,7 @@
       </c>
       <c r="G81" s="4"/>
       <c r="H81" s="4" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18298,7 +18295,7 @@
         <v>792</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E82" s="4"/>
       <c r="F82" s="4" t="n">
@@ -18306,7 +18303,7 @@
       </c>
       <c r="G82" s="4"/>
       <c r="H82" s="4" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18314,13 +18311,13 @@
         <v>80</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="C83" s="4" t="s">
         <v>792</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E83" s="4"/>
       <c r="F83" s="4" t="n">
@@ -18328,7 +18325,7 @@
       </c>
       <c r="G83" s="4"/>
       <c r="H83" s="4" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18336,7 +18333,7 @@
         <v>80</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>219</v>
@@ -18362,7 +18359,7 @@
         <v>792</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E85" s="4"/>
       <c r="F85" s="4" t="n">
@@ -18370,7 +18367,7 @@
       </c>
       <c r="G85" s="4"/>
       <c r="H85" s="4" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18384,7 +18381,7 @@
         <v>792</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E86" s="4"/>
       <c r="F86" s="4" t="n">
@@ -18392,7 +18389,7 @@
       </c>
       <c r="G86" s="4"/>
       <c r="H86" s="4" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18400,13 +18397,13 @@
         <v>80</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="C87" s="4" t="s">
         <v>792</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E87" s="4"/>
       <c r="F87" s="4" t="n">
@@ -18414,7 +18411,7 @@
       </c>
       <c r="G87" s="4"/>
       <c r="H87" s="4" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18428,7 +18425,7 @@
         <v>792</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E88" s="4"/>
       <c r="F88" s="4" t="n">
@@ -18436,7 +18433,7 @@
       </c>
       <c r="G88" s="4"/>
       <c r="H88" s="4" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18450,7 +18447,7 @@
         <v>792</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E89" s="4"/>
       <c r="F89" s="4" t="n">
@@ -18458,7 +18455,7 @@
       </c>
       <c r="G89" s="4"/>
       <c r="H89" s="4" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18472,7 +18469,7 @@
         <v>792</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E90" s="4"/>
       <c r="F90" s="4" t="n">
@@ -18480,7 +18477,7 @@
       </c>
       <c r="G90" s="4"/>
       <c r="H90" s="4" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18494,7 +18491,7 @@
         <v>792</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E91" s="4"/>
       <c r="F91" s="4" t="n">
@@ -18502,7 +18499,7 @@
       </c>
       <c r="G91" s="4"/>
       <c r="H91" s="4" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18516,17 +18513,17 @@
         <v>792</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E92" s="4"/>
       <c r="F92" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G92" s="4" t="s">
+        <v>848</v>
+      </c>
+      <c r="H92" s="4" t="s">
         <v>849</v>
-      </c>
-      <c r="H92" s="4" t="s">
-        <v>850</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18540,7 +18537,7 @@
         <v>792</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E93" s="4"/>
       <c r="F93" s="4" t="n">
@@ -18548,7 +18545,7 @@
       </c>
       <c r="G93" s="4"/>
       <c r="H93" s="4" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18562,7 +18559,7 @@
         <v>792</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E94" s="4"/>
       <c r="F94" s="4" t="n">
@@ -18570,7 +18567,7 @@
       </c>
       <c r="G94" s="4"/>
       <c r="H94" s="4" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18584,7 +18581,7 @@
         <v>792</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E95" s="4"/>
       <c r="F95" s="4" t="n">
@@ -18592,7 +18589,7 @@
       </c>
       <c r="G95" s="4"/>
       <c r="H95" s="4" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18606,7 +18603,7 @@
         <v>792</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E96" s="4"/>
       <c r="F96" s="4" t="n">
@@ -18614,7 +18611,7 @@
       </c>
       <c r="G96" s="4"/>
       <c r="H96" s="4" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18628,7 +18625,7 @@
         <v>792</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E97" s="4"/>
       <c r="F97" s="4" t="n">
@@ -18636,7 +18633,7 @@
       </c>
       <c r="G97" s="4"/>
       <c r="H97" s="4" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18650,7 +18647,7 @@
         <v>792</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E98" s="4"/>
       <c r="F98" s="4" t="n">
@@ -18658,7 +18655,7 @@
       </c>
       <c r="G98" s="4"/>
       <c r="H98" s="4" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18672,7 +18669,7 @@
         <v>792</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E99" s="4"/>
       <c r="F99" s="4" t="n">
@@ -18680,7 +18677,7 @@
       </c>
       <c r="G99" s="4"/>
       <c r="H99" s="4" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18694,7 +18691,7 @@
         <v>792</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E100" s="4"/>
       <c r="F100" s="4" t="n">
@@ -18702,7 +18699,7 @@
       </c>
       <c r="G100" s="4"/>
       <c r="H100" s="4" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18770,7 +18767,7 @@
         <v>80</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="C104" s="2" t="s">
         <v>219</v>
@@ -18790,7 +18787,7 @@
         <v>80</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="C105" s="2" t="s">
         <v>219</v>
@@ -18810,7 +18807,7 @@
         <v>80</v>
       </c>
       <c r="B106" s="7" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="C106" s="7" t="s">
         <v>219</v>
@@ -18823,7 +18820,7 @@
         <v>1</v>
       </c>
       <c r="G106" s="7" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="H106" s="7"/>
     </row>
@@ -18832,20 +18829,20 @@
         <v>80</v>
       </c>
       <c r="B107" s="7" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="C107" s="7" t="s">
+        <v>825</v>
+      </c>
+      <c r="D107" s="7" t="s">
         <v>826</v>
-      </c>
-      <c r="D107" s="7" t="s">
-        <v>827</v>
       </c>
       <c r="E107" s="7"/>
       <c r="F107" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G107" s="7" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="H107" s="7"/>
     </row>
@@ -18867,7 +18864,7 @@
         <v>1</v>
       </c>
       <c r="G108" s="7" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="H108" s="7"/>
     </row>
@@ -18896,7 +18893,7 @@
         <v>80</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="C110" s="2" t="s">
         <v>23</v>
@@ -18916,7 +18913,7 @@
         <v>80</v>
       </c>
       <c r="B111" s="7" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="C111" s="7" t="s">
         <v>23</v>
@@ -18929,7 +18926,7 @@
         <v>1</v>
       </c>
       <c r="G111" s="7" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="H111" s="7"/>
     </row>
@@ -18958,7 +18955,7 @@
         <v>80</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="C113" s="2" t="s">
         <v>23</v>
@@ -18978,7 +18975,7 @@
         <v>80</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="C114" s="2" t="s">
         <v>23</v>
@@ -18998,7 +18995,7 @@
         <v>80</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="C115" s="2" t="s">
         <v>23</v>
@@ -19018,7 +19015,7 @@
         <v>80</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="C116" s="2" t="s">
         <v>23</v>
@@ -19078,7 +19075,7 @@
         <v>80</v>
       </c>
       <c r="B119" s="7" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="C119" s="7" t="s">
         <v>23</v>
@@ -19091,7 +19088,7 @@
         <v>1</v>
       </c>
       <c r="G119" s="7" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="H119" s="7"/>
     </row>
@@ -19140,7 +19137,7 @@
         <v>80</v>
       </c>
       <c r="B122" s="7" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="C122" s="7" t="s">
         <v>23</v>
@@ -19153,7 +19150,7 @@
         <v>1</v>
       </c>
       <c r="G122" s="7" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="H122" s="7"/>
     </row>
@@ -19162,7 +19159,7 @@
         <v>80</v>
       </c>
       <c r="B123" s="7" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="C123" s="7" t="s">
         <v>23</v>
@@ -19175,7 +19172,7 @@
         <v>1</v>
       </c>
       <c r="G123" s="7" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="H123" s="7"/>
     </row>
@@ -19184,7 +19181,7 @@
         <v>80</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="C124" s="2" t="s">
         <v>23</v>
@@ -19224,7 +19221,7 @@
         <v>80</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="C126" s="2" t="s">
         <v>23</v>
@@ -19244,7 +19241,7 @@
         <v>80</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="C127" s="2" t="s">
         <v>23</v>
@@ -19277,7 +19274,7 @@
         <v>1</v>
       </c>
       <c r="G128" s="7" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="H128" s="7"/>
     </row>
@@ -19286,7 +19283,7 @@
         <v>80</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="C129" s="2" t="s">
         <v>23</v>
@@ -19315,7 +19312,7 @@
         <v>16</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="F130" s="2" t="n">
         <v>0</v>
@@ -19341,7 +19338,7 @@
         <v>1</v>
       </c>
       <c r="G131" s="7" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="H131" s="7"/>
     </row>
@@ -19423,7 +19420,7 @@
         <v>1</v>
       </c>
       <c r="G135" s="7" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="H135" s="7"/>
     </row>
@@ -19472,7 +19469,7 @@
         <v>286</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="C138" s="2" t="s">
         <v>23</v>
@@ -19492,7 +19489,7 @@
         <v>286</v>
       </c>
       <c r="B139" s="7" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="C139" s="7" t="s">
         <v>15</v>
@@ -19505,7 +19502,7 @@
         <v>1</v>
       </c>
       <c r="G139" s="7" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="H139" s="7"/>
     </row>
@@ -19514,7 +19511,7 @@
         <v>286</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="C140" s="2" t="s">
         <v>148</v>
@@ -19587,7 +19584,7 @@
         <v>1</v>
       </c>
       <c r="G143" s="7" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="H143" s="7"/>
     </row>
@@ -19596,7 +19593,7 @@
         <v>286</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="C144" s="2" t="s">
         <v>219</v>
@@ -19616,7 +19613,7 @@
         <v>286</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C145" s="2" t="s">
         <v>219</v>
@@ -19636,7 +19633,7 @@
         <v>286</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="C146" s="2" t="s">
         <v>219</v>
@@ -19656,7 +19653,7 @@
         <v>286</v>
       </c>
       <c r="B147" s="7" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C147" s="7" t="s">
         <v>219</v>
@@ -19669,7 +19666,7 @@
         <v>1</v>
       </c>
       <c r="G147" s="7" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="H147" s="7"/>
     </row>
@@ -19678,7 +19675,7 @@
         <v>286</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="C148" s="2" t="s">
         <v>219</v>
@@ -19798,7 +19795,7 @@
         <v>286</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="C154" s="2" t="s">
         <v>219</v>
@@ -19818,7 +19815,7 @@
         <v>286</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="C155" s="2" t="s">
         <v>219</v>
@@ -19871,7 +19868,7 @@
         <v>1</v>
       </c>
       <c r="G157" s="7" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="H157" s="7"/>
     </row>
@@ -20080,7 +20077,7 @@
         <v>286</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="C168" s="2" t="s">
         <v>23</v>
@@ -20100,7 +20097,7 @@
         <v>286</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="C169" s="2" t="s">
         <v>23</v>
@@ -20153,7 +20150,7 @@
         <v>1</v>
       </c>
       <c r="G171" s="7" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="H171" s="7"/>
     </row>
@@ -20162,7 +20159,7 @@
         <v>286</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="C172" s="2" t="s">
         <v>23</v>
@@ -20245,7 +20242,7 @@
         <v>650</v>
       </c>
       <c r="C176" s="7" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="D176" s="7" t="s">
         <v>24</v>
@@ -20255,7 +20252,7 @@
         <v>1</v>
       </c>
       <c r="G176" s="7" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="H176" s="7"/>
     </row>
@@ -20264,7 +20261,7 @@
         <v>286</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="C177" s="2" t="s">
         <v>23</v>
@@ -20284,7 +20281,7 @@
         <v>286</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="C178" s="2" t="s">
         <v>23</v>
@@ -20304,7 +20301,7 @@
         <v>286</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="C179" s="2" t="s">
         <v>23</v>
@@ -20324,7 +20321,7 @@
         <v>286</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="C180" s="2" t="s">
         <v>23</v>
@@ -20344,7 +20341,7 @@
         <v>286</v>
       </c>
       <c r="B181" s="7" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="C181" s="7" t="s">
         <v>23</v>
@@ -20357,7 +20354,7 @@
         <v>1</v>
       </c>
       <c r="G181" s="7" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="H181" s="7"/>
     </row>
@@ -20366,7 +20363,7 @@
         <v>286</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="C182" s="2" t="s">
         <v>23</v>
@@ -20386,10 +20383,10 @@
         <v>286</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="D183" s="2" t="s">
         <v>24</v>
@@ -20406,7 +20403,7 @@
         <v>286</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="C184" s="2" t="s">
         <v>23</v>
@@ -20426,7 +20423,7 @@
         <v>286</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="C185" s="2" t="s">
         <v>23</v>
@@ -20506,7 +20503,7 @@
         <v>286</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="C189" s="2" t="s">
         <v>23</v>
@@ -20526,7 +20523,7 @@
         <v>286</v>
       </c>
       <c r="B190" s="7" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="C190" s="7" t="s">
         <v>23</v>
@@ -20539,7 +20536,7 @@
         <v>1</v>
       </c>
       <c r="G190" s="7" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="H190" s="7"/>
     </row>
@@ -20561,7 +20558,7 @@
         <v>1</v>
       </c>
       <c r="G191" s="7" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="H191" s="7"/>
     </row>
@@ -20613,7 +20610,7 @@
         <v>257</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="D194" s="2" t="s">
         <v>24</v>
@@ -20643,7 +20640,7 @@
         <v>1</v>
       </c>
       <c r="G195" s="7" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="H195" s="7"/>
     </row>
@@ -20652,7 +20649,7 @@
         <v>286</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="C196" s="2" t="s">
         <v>23</v>
@@ -20672,7 +20669,7 @@
         <v>286</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="C197" s="2" t="s">
         <v>23</v>
@@ -20692,7 +20689,7 @@
         <v>286</v>
       </c>
       <c r="B198" s="7" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="C198" s="7" t="s">
         <v>23</v>
@@ -20705,7 +20702,7 @@
         <v>1</v>
       </c>
       <c r="G198" s="7" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="H198" s="7"/>
     </row>
@@ -20714,7 +20711,7 @@
         <v>286</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="C199" s="2" t="s">
         <v>23</v>
@@ -20754,7 +20751,7 @@
         <v>286</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="C201" s="2" t="s">
         <v>23</v>
@@ -20774,7 +20771,7 @@
         <v>286</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="C202" s="2" t="s">
         <v>23</v>
@@ -20794,7 +20791,7 @@
         <v>286</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="C203" s="2" t="s">
         <v>23</v>
@@ -20823,7 +20820,7 @@
         <v>792</v>
       </c>
       <c r="E204" s="2" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="F204" s="2" t="n">
         <v>0</v>
@@ -20845,7 +20842,7 @@
         <v>792</v>
       </c>
       <c r="E205" s="2" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="F205" s="2" t="n">
         <v>0</v>
@@ -20867,7 +20864,7 @@
         <v>794</v>
       </c>
       <c r="E206" s="6" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="F206" s="6" t="n">
         <v>0</v>
@@ -20891,7 +20888,7 @@
         <v>792</v>
       </c>
       <c r="E207" s="2" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="F207" s="2" t="n">
         <v>0</v>
@@ -20913,7 +20910,7 @@
         <v>792</v>
       </c>
       <c r="E208" s="2" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="F208" s="2" t="n">
         <v>0</v>
@@ -20935,7 +20932,7 @@
         <v>794</v>
       </c>
       <c r="E209" s="6" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="F209" s="6" t="n">
         <v>0</v>
@@ -20959,7 +20956,7 @@
         <v>792</v>
       </c>
       <c r="E210" s="2" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="F210" s="2" t="n">
         <v>0</v>
@@ -20981,7 +20978,7 @@
         <v>792</v>
       </c>
       <c r="E211" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F211" s="2" t="n">
         <v>0</v>
@@ -21003,7 +21000,7 @@
         <v>792</v>
       </c>
       <c r="E212" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F212" s="2" t="n">
         <v>0</v>
@@ -21025,7 +21022,7 @@
         <v>792</v>
       </c>
       <c r="E213" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F213" s="2" t="n">
         <v>0</v>
@@ -21047,13 +21044,13 @@
         <v>792</v>
       </c>
       <c r="E214" s="7" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F214" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G214" s="7" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="H214" s="7"/>
     </row>
@@ -21071,7 +21068,7 @@
         <v>792</v>
       </c>
       <c r="E215" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F215" s="2" t="n">
         <v>0</v>
@@ -21093,7 +21090,7 @@
         <v>792</v>
       </c>
       <c r="E216" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F216" s="2" t="n">
         <v>0</v>
@@ -21106,7 +21103,7 @@
         <v>473</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="C217" s="2" t="s">
         <v>219</v>
@@ -21115,7 +21112,7 @@
         <v>792</v>
       </c>
       <c r="E217" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F217" s="2" t="n">
         <v>0</v>
@@ -21159,7 +21156,7 @@
         <v>792</v>
       </c>
       <c r="E219" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F219" s="2" t="n">
         <v>0</v>
@@ -21181,7 +21178,7 @@
         <v>792</v>
       </c>
       <c r="E220" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F220" s="2" t="n">
         <v>0</v>
@@ -21203,7 +21200,7 @@
         <v>792</v>
       </c>
       <c r="E221" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F221" s="2" t="n">
         <v>0</v>
@@ -21225,7 +21222,7 @@
         <v>792</v>
       </c>
       <c r="E222" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F222" s="2" t="n">
         <v>0</v>
@@ -21247,7 +21244,7 @@
         <v>792</v>
       </c>
       <c r="E223" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F223" s="2" t="n">
         <v>0</v>
@@ -21260,7 +21257,7 @@
         <v>473</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="C224" s="2" t="s">
         <v>219</v>
@@ -21269,7 +21266,7 @@
         <v>792</v>
       </c>
       <c r="E224" s="2" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="F224" s="2" t="n">
         <v>0</v>
@@ -21282,7 +21279,7 @@
         <v>473</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="C225" s="2" t="s">
         <v>219</v>
@@ -21291,7 +21288,7 @@
         <v>792</v>
       </c>
       <c r="E225" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F225" s="2" t="n">
         <v>0</v>
@@ -21304,7 +21301,7 @@
         <v>473</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="C226" s="2" t="s">
         <v>219</v>
@@ -21313,7 +21310,7 @@
         <v>792</v>
       </c>
       <c r="E226" s="2" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="F226" s="2" t="n">
         <v>0</v>
@@ -21326,7 +21323,7 @@
         <v>473</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="C227" s="2" t="s">
         <v>219</v>
@@ -21426,7 +21423,7 @@
         <v>473</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="C232" s="2" t="s">
         <v>219</v>
@@ -21446,7 +21443,7 @@
         <v>473</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="C233" s="2" t="s">
         <v>219</v>
@@ -21466,7 +21463,7 @@
         <v>473</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="C234" s="2" t="s">
         <v>219</v>
@@ -21486,7 +21483,7 @@
         <v>473</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="C235" s="2" t="s">
         <v>219</v>
@@ -21506,7 +21503,7 @@
         <v>473</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="C236" s="2" t="s">
         <v>219</v>
@@ -21555,7 +21552,7 @@
         <v>794</v>
       </c>
       <c r="E238" s="6" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="F238" s="6" t="n">
         <v>0</v>
@@ -21576,7 +21573,7 @@
         <v>16</v>
       </c>
       <c r="D239" s="2" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="E239" s="2"/>
       <c r="F239" s="2" t="n">
@@ -21610,7 +21607,7 @@
         <v>473</v>
       </c>
       <c r="B241" s="7" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="C241" s="7" t="s">
         <v>219</v>
@@ -21623,7 +21620,7 @@
         <v>1</v>
       </c>
       <c r="G241" s="7" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="H241" s="7"/>
     </row>
@@ -21632,7 +21629,7 @@
         <v>473</v>
       </c>
       <c r="B242" s="2" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="C242" s="2" t="s">
         <v>23</v>
@@ -21652,7 +21649,7 @@
         <v>473</v>
       </c>
       <c r="B243" s="2" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="C243" s="2" t="s">
         <v>219</v>
@@ -21672,7 +21669,7 @@
         <v>473</v>
       </c>
       <c r="B244" s="2" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C244" s="2" t="s">
         <v>219</v>
@@ -21692,7 +21689,7 @@
         <v>473</v>
       </c>
       <c r="B245" s="2" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="C245" s="2" t="s">
         <v>219</v>
@@ -21712,7 +21709,7 @@
         <v>473</v>
       </c>
       <c r="B246" s="2" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="C246" s="2" t="s">
         <v>219</v>
@@ -21732,7 +21729,7 @@
         <v>473</v>
       </c>
       <c r="B247" s="2" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C247" s="2" t="s">
         <v>219</v>
@@ -21752,7 +21749,7 @@
         <v>473</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="C248" s="2" t="s">
         <v>219</v>
@@ -21772,7 +21769,7 @@
         <v>473</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="C249" s="2" t="s">
         <v>219</v>
@@ -21792,7 +21789,7 @@
         <v>473</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="C250" s="2" t="s">
         <v>219</v>
@@ -21812,7 +21809,7 @@
         <v>473</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="C251" s="2" t="s">
         <v>219</v>
@@ -21832,7 +21829,7 @@
         <v>473</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="C252" s="2" t="s">
         <v>219</v>
@@ -21852,7 +21849,7 @@
         <v>473</v>
       </c>
       <c r="B253" s="2" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="C253" s="2" t="s">
         <v>219</v>
@@ -21872,7 +21869,7 @@
         <v>473</v>
       </c>
       <c r="B254" s="7" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="C254" s="7" t="s">
         <v>219</v>
@@ -21885,7 +21882,7 @@
         <v>1</v>
       </c>
       <c r="G254" s="7" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="H254" s="7"/>
     </row>
@@ -21894,7 +21891,7 @@
         <v>473</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="C255" s="2" t="s">
         <v>219</v>
@@ -21934,7 +21931,7 @@
         <v>473</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="C257" s="2" t="s">
         <v>219</v>
@@ -22034,7 +22031,7 @@
         <v>473</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="C262" s="2" t="s">
         <v>219</v>
@@ -22054,7 +22051,7 @@
         <v>473</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="C263" s="2" t="s">
         <v>219</v>
@@ -22074,7 +22071,7 @@
         <v>473</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="C264" s="2" t="s">
         <v>219</v>
@@ -22154,7 +22151,7 @@
         <v>473</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="C268" s="2" t="s">
         <v>219</v>
@@ -22294,7 +22291,7 @@
         <v>473</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="C275" s="2" t="s">
         <v>219</v>
@@ -22414,7 +22411,7 @@
         <v>473</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="C281" s="2" t="s">
         <v>219</v>
@@ -22454,7 +22451,7 @@
         <v>473</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="C283" s="2" t="s">
         <v>219</v>
@@ -22514,7 +22511,7 @@
         <v>473</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="C286" s="2" t="s">
         <v>219</v>
@@ -22547,7 +22544,7 @@
         <v>1</v>
       </c>
       <c r="G287" s="7" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="H287" s="7"/>
     </row>
@@ -22616,7 +22613,7 @@
         <v>473</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="C291" s="2" t="s">
         <v>15</v>
@@ -22625,7 +22622,7 @@
         <v>16</v>
       </c>
       <c r="E291" s="2" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="F291" s="2" t="n">
         <v>0</v>
@@ -22698,7 +22695,7 @@
         <v>473</v>
       </c>
       <c r="B295" s="2" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="C295" s="2" t="s">
         <v>219</v>
@@ -22738,7 +22735,7 @@
         <v>473</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="C297" s="2" t="s">
         <v>219</v>
@@ -22818,7 +22815,7 @@
         <v>473</v>
       </c>
       <c r="B301" s="2" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="C301" s="2" t="s">
         <v>219</v>
@@ -22851,7 +22848,7 @@
         <v>1</v>
       </c>
       <c r="G302" s="7" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="H302" s="7"/>
     </row>
@@ -22860,7 +22857,7 @@
         <v>473</v>
       </c>
       <c r="B303" s="2" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="C303" s="2" t="s">
         <v>219</v>
@@ -22880,7 +22877,7 @@
         <v>473</v>
       </c>
       <c r="B304" s="2" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="C304" s="2" t="s">
         <v>219</v>
@@ -22900,7 +22897,7 @@
         <v>473</v>
       </c>
       <c r="B305" s="2" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="C305" s="2" t="s">
         <v>219</v>
@@ -22920,7 +22917,7 @@
         <v>473</v>
       </c>
       <c r="B306" s="2" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="C306" s="2" t="s">
         <v>219</v>
@@ -22940,7 +22937,7 @@
         <v>473</v>
       </c>
       <c r="B307" s="2" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="C307" s="2" t="s">
         <v>219</v>
@@ -22960,7 +22957,7 @@
         <v>473</v>
       </c>
       <c r="B308" s="2" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="C308" s="2" t="s">
         <v>219</v>
@@ -22980,7 +22977,7 @@
         <v>473</v>
       </c>
       <c r="B309" s="2" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="C309" s="2" t="s">
         <v>219</v>
@@ -23000,7 +22997,7 @@
         <v>473</v>
       </c>
       <c r="B310" s="2" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C310" s="2" t="s">
         <v>219</v>
@@ -23020,7 +23017,7 @@
         <v>473</v>
       </c>
       <c r="B311" s="2" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="C311" s="2" t="s">
         <v>219</v>
@@ -23040,7 +23037,7 @@
         <v>473</v>
       </c>
       <c r="B312" s="2" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="C312" s="2" t="s">
         <v>219</v>
@@ -23060,7 +23057,7 @@
         <v>473</v>
       </c>
       <c r="B313" s="2" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="C313" s="2" t="s">
         <v>219</v>
@@ -23080,7 +23077,7 @@
         <v>473</v>
       </c>
       <c r="B314" s="2" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="C314" s="2" t="s">
         <v>219</v>
@@ -23100,7 +23097,7 @@
         <v>473</v>
       </c>
       <c r="B315" s="2" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="C315" s="2" t="s">
         <v>219</v>
@@ -23120,7 +23117,7 @@
         <v>473</v>
       </c>
       <c r="B316" s="2" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="C316" s="2" t="s">
         <v>219</v>
@@ -23140,7 +23137,7 @@
         <v>473</v>
       </c>
       <c r="B317" s="2" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="C317" s="2" t="s">
         <v>219</v>
@@ -23160,7 +23157,7 @@
         <v>473</v>
       </c>
       <c r="B318" s="7" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="C318" s="7" t="s">
         <v>219</v>
@@ -23173,7 +23170,7 @@
         <v>1</v>
       </c>
       <c r="G318" s="7" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="H318" s="7"/>
     </row>
@@ -23182,7 +23179,7 @@
         <v>473</v>
       </c>
       <c r="B319" s="2" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="C319" s="2" t="s">
         <v>219</v>
@@ -23202,7 +23199,7 @@
         <v>473</v>
       </c>
       <c r="B320" s="2" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="C320" s="2" t="s">
         <v>219</v>
@@ -23222,7 +23219,7 @@
         <v>473</v>
       </c>
       <c r="B321" s="2" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="C321" s="2" t="s">
         <v>23</v>
@@ -23242,7 +23239,7 @@
         <v>473</v>
       </c>
       <c r="B322" s="2" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="C322" s="2" t="s">
         <v>219</v>
@@ -23262,7 +23259,7 @@
         <v>473</v>
       </c>
       <c r="B323" s="7" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="C323" s="7" t="s">
         <v>219</v>
@@ -23275,7 +23272,7 @@
         <v>1</v>
       </c>
       <c r="G323" s="7" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="H323" s="7"/>
     </row>
@@ -23284,7 +23281,7 @@
         <v>473</v>
       </c>
       <c r="B324" s="2" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="C324" s="2" t="s">
         <v>23</v>
@@ -23304,7 +23301,7 @@
         <v>473</v>
       </c>
       <c r="B325" s="2" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="C325" s="2" t="s">
         <v>219</v>
@@ -23324,7 +23321,7 @@
         <v>473</v>
       </c>
       <c r="B326" s="2" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="C326" s="2" t="s">
         <v>23</v>
@@ -23344,7 +23341,7 @@
         <v>473</v>
       </c>
       <c r="B327" s="2" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="C327" s="2" t="s">
         <v>219</v>
@@ -23364,7 +23361,7 @@
         <v>473</v>
       </c>
       <c r="B328" s="7" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="C328" s="7" t="s">
         <v>219</v>
@@ -23377,7 +23374,7 @@
         <v>1</v>
       </c>
       <c r="G328" s="7" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="H328" s="7"/>
     </row>
@@ -23386,7 +23383,7 @@
         <v>473</v>
       </c>
       <c r="B329" s="2" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="C329" s="2" t="s">
         <v>219</v>
@@ -23406,7 +23403,7 @@
         <v>473</v>
       </c>
       <c r="B330" s="2" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="C330" s="2" t="s">
         <v>219</v>
@@ -23426,7 +23423,7 @@
         <v>473</v>
       </c>
       <c r="B331" s="2" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="C331" s="2" t="s">
         <v>219</v>
@@ -23446,7 +23443,7 @@
         <v>473</v>
       </c>
       <c r="B332" s="2" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="C332" s="2" t="s">
         <v>219</v>
@@ -23466,7 +23463,7 @@
         <v>473</v>
       </c>
       <c r="B333" s="2" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="C333" s="2" t="s">
         <v>219</v>
@@ -23486,7 +23483,7 @@
         <v>473</v>
       </c>
       <c r="B334" s="2" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="C334" s="2" t="s">
         <v>219</v>
@@ -23506,7 +23503,7 @@
         <v>473</v>
       </c>
       <c r="B335" s="2" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="C335" s="2" t="s">
         <v>219</v>
@@ -23526,7 +23523,7 @@
         <v>473</v>
       </c>
       <c r="B336" s="2" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="C336" s="2" t="s">
         <v>219</v>
@@ -23546,7 +23543,7 @@
         <v>473</v>
       </c>
       <c r="B337" s="2" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="C337" s="2" t="s">
         <v>219</v>
@@ -23566,7 +23563,7 @@
         <v>473</v>
       </c>
       <c r="B338" s="6" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="C338" s="6" t="s">
         <v>793</v>
@@ -23575,7 +23572,7 @@
         <v>794</v>
       </c>
       <c r="E338" s="6" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="F338" s="6" t="n">
         <v>0</v>
@@ -23590,7 +23587,7 @@
         <v>473</v>
       </c>
       <c r="B339" s="2" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="C339" s="2" t="s">
         <v>219</v>
@@ -23610,7 +23607,7 @@
         <v>473</v>
       </c>
       <c r="B340" s="2" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="C340" s="2" t="s">
         <v>219</v>
@@ -23630,7 +23627,7 @@
         <v>473</v>
       </c>
       <c r="B341" s="2" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="C341" s="2" t="s">
         <v>23</v>
@@ -23650,7 +23647,7 @@
         <v>473</v>
       </c>
       <c r="B342" s="2" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="C342" s="2" t="s">
         <v>219</v>
@@ -23670,7 +23667,7 @@
         <v>473</v>
       </c>
       <c r="B343" s="2" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="C343" s="2" t="s">
         <v>219</v>
@@ -23690,7 +23687,7 @@
         <v>473</v>
       </c>
       <c r="B344" s="2" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="C344" s="2" t="s">
         <v>219</v>
@@ -23710,7 +23707,7 @@
         <v>473</v>
       </c>
       <c r="B345" s="2" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="C345" s="2" t="s">
         <v>219</v>
@@ -23730,7 +23727,7 @@
         <v>473</v>
       </c>
       <c r="B346" s="2" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="C346" s="2" t="s">
         <v>219</v>
@@ -23750,7 +23747,7 @@
         <v>473</v>
       </c>
       <c r="B347" s="2" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="C347" s="2" t="s">
         <v>219</v>
@@ -23770,7 +23767,7 @@
         <v>473</v>
       </c>
       <c r="B348" s="2" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="C348" s="2" t="s">
         <v>219</v>
@@ -23790,7 +23787,7 @@
         <v>473</v>
       </c>
       <c r="B349" s="2" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="C349" s="2" t="s">
         <v>219</v>
@@ -23810,7 +23807,7 @@
         <v>473</v>
       </c>
       <c r="B350" s="2" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="C350" s="2" t="s">
         <v>219</v>
@@ -23830,7 +23827,7 @@
         <v>473</v>
       </c>
       <c r="B351" s="2" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="C351" s="2" t="s">
         <v>219</v>
@@ -23850,7 +23847,7 @@
         <v>473</v>
       </c>
       <c r="B352" s="2" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="C352" s="2" t="s">
         <v>219</v>
@@ -23870,7 +23867,7 @@
         <v>473</v>
       </c>
       <c r="B353" s="2" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="C353" s="2" t="s">
         <v>219</v>
@@ -23890,7 +23887,7 @@
         <v>473</v>
       </c>
       <c r="B354" s="2" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="C354" s="2" t="s">
         <v>219</v>
@@ -23910,7 +23907,7 @@
         <v>473</v>
       </c>
       <c r="B355" s="2" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="C355" s="2" t="s">
         <v>219</v>
@@ -23930,7 +23927,7 @@
         <v>473</v>
       </c>
       <c r="B356" s="2" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="C356" s="2" t="s">
         <v>219</v>
@@ -23950,7 +23947,7 @@
         <v>473</v>
       </c>
       <c r="B357" s="2" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="C357" s="2" t="s">
         <v>219</v>
@@ -23970,7 +23967,7 @@
         <v>473</v>
       </c>
       <c r="B358" s="2" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="C358" s="2" t="s">
         <v>23</v>
@@ -23990,7 +23987,7 @@
         <v>473</v>
       </c>
       <c r="B359" s="2" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="C359" s="2" t="s">
         <v>23</v>
@@ -24010,7 +24007,7 @@
         <v>473</v>
       </c>
       <c r="B360" s="2" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C360" s="2" t="s">
         <v>219</v>
@@ -24030,7 +24027,7 @@
         <v>473</v>
       </c>
       <c r="B361" s="2" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="C361" s="2" t="s">
         <v>219</v>
@@ -24050,7 +24047,7 @@
         <v>473</v>
       </c>
       <c r="B362" s="2" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="C362" s="2" t="s">
         <v>219</v>
@@ -24114,7 +24111,7 @@
         <v>7</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24125,10 +24122,10 @@
         <v>10</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>997</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>998</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>999</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>15</v>
@@ -24137,7 +24134,7 @@
         <v>16</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24151,16 +24148,16 @@
         <v>177</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>1000</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>1001</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>1002</v>
-      </c>
       <c r="F3" s="2" t="s">
         <v>24</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24174,16 +24171,16 @@
         <v>177</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>24</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24197,16 +24194,16 @@
         <v>168</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>24</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24220,16 +24217,16 @@
         <v>168</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>24</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24243,16 +24240,16 @@
         <v>168</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>24</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
     </row>
   </sheetData>
@@ -24282,10 +24279,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>1007</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>1008</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24294,7 +24291,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTA('200V Devices'!C2:C393)</f>
@@ -24303,7 +24300,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF('200V Devices'!I2:I393,"Done (pilot)")</f>
@@ -24312,7 +24309,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF('200V Devices'!I2:I393,"To do")</f>
@@ -24321,7 +24318,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF('200V Devices'!J2:J393,"Matched from 200V tab")</f>
@@ -24330,7 +24327,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTA('Not found'!C2:C7)</f>
@@ -24339,7 +24336,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">B3+B7</f>
@@ -24352,10 +24349,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>1015</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>1016</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24409,29 +24406,29 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="B17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B18" s="9" t="s">
         <v>1018</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>1019</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
+        <v>1019</v>
+      </c>
+      <c r="B19" s="9" t="s">
         <v>1020</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>1021</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="B21" s="9" t="n">
         <f aca="false">COUNTA('Ports without device'!A2:A362)</f>
@@ -24440,7 +24437,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="B22" s="9" t="n">
         <f aca="false">COUNTIF('Ports without device'!F2:F362,"&gt;0")</f>
@@ -24449,7 +24446,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="B23" s="9" t="n">
         <f aca="false">COUNTIF('Ports without device'!F2:F362,0)</f>
@@ -24458,7 +24455,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="B24" s="9" t="n">
         <f aca="false">COUNTIF('Ports without device'!H2:H362,"Pilot staff outlet*")</f>
@@ -24467,7 +24464,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="B25" s="9" t="n">
         <f aca="false">COUNTIF('Ports without device'!C2:C362,"None (tagged only)")</f>
@@ -24476,10 +24473,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
+        <v>1026</v>
+      </c>
+      <c r="B26" s="9" t="s">
         <v>1027</v>
-      </c>
-      <c r="B26" s="9" t="s">
-        <v>1028</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Review tab: lv6 spanning-tree limit and STP on 2600/2700
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZ7jJsE6GWKm6ehHY39VNr
</commit_message>
<xml_diff>
--- a/200V Device Port List.xlsx
+++ b/200V Device Port List.xlsx
@@ -630,13 +630,25 @@
     <t xml:space="preserve">6</t>
   </si>
   <si>
-    <t xml:space="preserve">VLANs 2600 and 2700 have no spanning-tree</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other VLANs on lv6, and 2600/2700 on lv3 and lv4, have spanning-tree enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add spanning-tree to 2600 and 2700 on lv6</t>
+    <t xml:space="preserve">Raise spanning-tree limit, then enable spanning-tree on 2600 and 2700</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lv6 has 35 VLANs but spanning-tree on only 32, the ICX default maximum, so 2600 (CCTV), 2700 (AV) and 2953 run without spanning-tree. lv4 already has system-max spanning-tree 40 configured but still shows 32, which suggests the new limit only applies after a reload</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run on lv6:
+configure terminal
+system-max spanning-tree 128
+write memory
+Then reload in a maintenance window, then:
+configure terminal
+vlan 2600
+ spanning-tree
+ exit
+vlan 2700
+ spanning-tree
+ exit
+write memory</t>
   </si>
   <si>
     <t xml:space="preserve">VLAN 100 tagged on every port (1/1/1-1/1/12)</t>
@@ -6192,7 +6204,7 @@
       <c r="H89" s="4"/>
       <c r="I89" s="4"/>
     </row>
-    <row r="90" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="5" t="n">
         <v>80</v>
       </c>

</xml_diff>

<commit_message>
Remove mentions of the LT2-1 trunk VLAN tagging
Drops the prerequisite row from the change document and the 6 Oct
tagging notes from the Switches and Ports without device tabs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZ7jJsE6GWKm6ehHY39VNr
</commit_message>
<xml_diff>
--- a/200V Device Port List.xlsx
+++ b/200V Device Port List.xlsx
@@ -2900,7 +2900,7 @@
     <t xml:space="preserve">10_F0_68_0C_06_D6</t>
   </si>
   <si>
-    <t xml:space="preserve">Via LT2-1 port 1/1/23 (their 1/1/12), confirmed by LLDP. New VLANs tagged on LT2-1 1/1/23 on 6 Oct 2026</t>
+    <t xml:space="preserve">Via LT2-1 port 1/1/23 (their 1/1/12), confirmed by LLDP</t>
   </si>
   <si>
     <t xml:space="preserve">192.168.122.13</t>
@@ -2909,7 +2909,7 @@
     <t xml:space="preserve">10_F0_68_0B_D2_3E</t>
   </si>
   <si>
-    <t xml:space="preserve">Via LT2-1 port 1/1/24 (their 1/1/12), confirmed by LLDP. New VLANs tagged on LT2-1 1/1/24 on 6 Oct 2026</t>
+    <t xml:space="preserve">Via LT2-1 port 1/1/24 (their 1/1/12), confirmed by LLDP</t>
   </si>
   <si>
     <t xml:space="preserve">192.168.122.14</t>
@@ -2987,13 +2987,13 @@
     <t xml:space="preserve">10:F0:68:0C:06:E1, 10:F0:68:0C:06:D6</t>
   </si>
   <si>
-    <t xml:space="preserve">Uplink to switch-200V-LT2-2 (LLDP). 22 new VLANs (2000-2953) tagged 6 Oct 2026, ahead of cutover</t>
+    <t xml:space="preserve">Uplink to switch-200V-LT2-2 (LLDP)</t>
   </si>
   <si>
     <t xml:space="preserve">10:F0:68:0B:D2:49, 10:F0:68:0B:D2:3E, AC:B4:80:F1:61:7F</t>
   </si>
   <si>
-    <t xml:space="preserve">Uplink to switch-200V-LT2-3 (LLDP). 22 new VLANs (2000-2953) tagged 6 Oct 2026, ahead of cutover</t>
+    <t xml:space="preserve">Uplink to switch-200V-LT2-3 (LLDP)</t>
   </si>
   <si>
     <t xml:space="preserve">1212,1213,1230,1250,1271,1272,1273,2000,2010,2020,2100,2200,2300,2310,2320,2400,2500,2510,2520,2530,2600,2700,2800,2810,2900,2950,2951,2952,2953</t>

</xml_diff>

<commit_message>
Add config to move 13 AV outlets (20:7B:D2:30 devices) from 1230 to 2700
Ports from the Dycom patching sheet (2025-07-30): lv3 7 ports, lv4 6
ports, all untagged 1230 with no listed device. Noted on the Ports
without device tab.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZ7jJsE6GWKm6ehHY39VNr
</commit_message>
<xml_diff>
--- a/200V Device Port List.xlsx
+++ b/200V Device Port List.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6083" uniqueCount="1284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6096" uniqueCount="1297">
   <si>
     <t xml:space="preserve">200V migration: items for review</t>
   </si>
@@ -3323,6 +3323,9 @@
     <t xml:space="preserve">Moved to 2700 on 9 Oct (unlisted AV device).</t>
   </si>
   <si>
+    <t xml:space="preserve">AV outlet 200V3J5, device 20:7B:D2:30:98:F3 (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+  </si>
+  <si>
     <t xml:space="preserve">D8:43:AE:B1:6E:9B</t>
   </si>
   <si>
@@ -3446,6 +3449,9 @@
     <t xml:space="preserve">D8:43:AE:B1:6C:A8</t>
   </si>
   <si>
+    <t xml:space="preserve">AV outlet 200V3G16, device 20:7B:D2:30:98:D6 (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+  </si>
+  <si>
     <t xml:space="preserve">4/1/45</t>
   </si>
   <si>
@@ -3461,18 +3467,30 @@
     <t xml:space="preserve">5/1/11</t>
   </si>
   <si>
+    <t xml:space="preserve">AV outlet 200V3H2, device 20:7B:D2:30:99:09 (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+  </si>
+  <si>
     <t xml:space="preserve">D8:43:AE:B1:6E:B0</t>
   </si>
   <si>
+    <t xml:space="preserve">AV outlet 200V3I8, device 20:7B:D2:30:98:AF (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+  </si>
+  <si>
     <t xml:space="preserve">D8:43:AE:B1:6E:3C</t>
   </si>
   <si>
     <t xml:space="preserve">D8:43:AE:B1:6F:04</t>
   </si>
   <si>
+    <t xml:space="preserve">AV outlet 200V3I16, device 20:7B:D2:30:98:D2 (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+  </si>
+  <si>
     <t xml:space="preserve">5/1/40</t>
   </si>
   <si>
+    <t xml:space="preserve">AV outlet 200V3H14, device 20:7B:D2:30:98:B1 (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+  </si>
+  <si>
     <t xml:space="preserve">5/1/43</t>
   </si>
   <si>
@@ -3482,15 +3500,30 @@
     <t xml:space="preserve">5/1/47</t>
   </si>
   <si>
+    <t xml:space="preserve">AV outlet 200V3H21, device 20:7B:D2:30:99:29 (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+  </si>
+  <si>
     <t xml:space="preserve">1272,1273,2300,2310,2311,2320,2321</t>
   </si>
   <si>
     <t xml:space="preserve">D8:43:AE:B1:6E:06</t>
   </si>
   <si>
+    <t xml:space="preserve">AV outlet 200V4H22, device 20:7B:D2:30:98:FD (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AV outlet 200V4I10, device 20:7B:D2:30:98:EF (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+  </si>
+  <si>
     <t xml:space="preserve">D8:43:AE:B1:6A:29</t>
   </si>
   <si>
+    <t xml:space="preserve">AV outlet 200V4J4, device 20:7B:D2:30:98:DB (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AV outlet 200V4J14, device 20:7B:D2:30:99:0E (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+  </si>
+  <si>
     <t xml:space="preserve">00:09:F5:32:D9:F7</t>
   </si>
   <si>
@@ -3515,6 +3548,9 @@
     <t xml:space="preserve">A0:4A:5E:E7:D5:71</t>
   </si>
   <si>
+    <t xml:space="preserve">AV outlet 200V4F5, device 20:7B:D2:30:98:DF (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+  </si>
+  <si>
     <t xml:space="preserve">D8:43:AE:B1:6D:56</t>
   </si>
   <si>
@@ -3522,6 +3558,9 @@
   </si>
   <si>
     <t xml:space="preserve">38:4B:76:E0:B0:B1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AV outlet 200V4H2, device 20:7B:D2:30:98:C2 (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
   </si>
   <si>
     <t xml:space="preserve">F8:25:51:CC:2C:76</t>
@@ -21843,7 +21882,9 @@
         <v>0</v>
       </c>
       <c r="G57" s="13"/>
-      <c r="H57" s="13"/>
+      <c r="H57" s="13" t="s">
+        <v>1091</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="13" t="s">
@@ -21903,7 +21944,7 @@
         <v>1</v>
       </c>
       <c r="G60" s="11" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="H60" s="11" t="s">
         <v>1090</v>
@@ -21934,7 +21975,7 @@
         <v>95</v>
       </c>
       <c r="B62" s="13" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="C62" s="13" t="s">
         <v>495</v>
@@ -21967,7 +22008,7 @@
         <v>1</v>
       </c>
       <c r="G63" s="11" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="H63" s="11" t="s">
         <v>1080</v>
@@ -21998,7 +22039,7 @@
         <v>95</v>
       </c>
       <c r="B65" s="13" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="C65" s="13" t="s">
         <v>495</v>
@@ -22161,10 +22202,10 @@
         <v>145</v>
       </c>
       <c r="C73" s="13" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="E73" s="13"/>
       <c r="F73" s="13" t="n">
@@ -22181,17 +22222,17 @@
         <v>108</v>
       </c>
       <c r="C74" s="11" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="D74" s="11" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="E74" s="11"/>
       <c r="F74" s="11" t="n">
         <v>1</v>
       </c>
       <c r="G74" s="11" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="H74" s="11" t="s">
         <v>1080</v>
@@ -22215,7 +22256,7 @@
         <v>1</v>
       </c>
       <c r="G75" s="11" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="H75" s="11" t="s">
         <v>1080</v>
@@ -22239,7 +22280,7 @@
         <v>1</v>
       </c>
       <c r="G76" s="11" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="H76" s="11" t="s">
         <v>1080</v>
@@ -22263,7 +22304,7 @@
         <v>1</v>
       </c>
       <c r="G77" s="11" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="H77" s="11" t="s">
         <v>1080</v>
@@ -22280,7 +22321,7 @@
         <v>1062</v>
       </c>
       <c r="D78" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E78" s="11"/>
       <c r="F78" s="11" t="n">
@@ -22288,7 +22329,7 @@
       </c>
       <c r="G78" s="11"/>
       <c r="H78" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22302,7 +22343,7 @@
         <v>1062</v>
       </c>
       <c r="D79" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E79" s="11"/>
       <c r="F79" s="11" t="n">
@@ -22310,7 +22351,7 @@
       </c>
       <c r="G79" s="11"/>
       <c r="H79" s="11" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22324,7 +22365,7 @@
         <v>1062</v>
       </c>
       <c r="D80" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E80" s="11"/>
       <c r="F80" s="11" t="n">
@@ -22332,7 +22373,7 @@
       </c>
       <c r="G80" s="11"/>
       <c r="H80" s="11" t="s">
-        <v>1104</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22346,7 +22387,7 @@
         <v>1062</v>
       </c>
       <c r="D81" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E81" s="11"/>
       <c r="F81" s="11" t="n">
@@ -22354,7 +22395,7 @@
       </c>
       <c r="G81" s="11"/>
       <c r="H81" s="11" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22368,7 +22409,7 @@
         <v>1062</v>
       </c>
       <c r="D82" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E82" s="11"/>
       <c r="F82" s="11" t="n">
@@ -22376,7 +22417,7 @@
       </c>
       <c r="G82" s="11"/>
       <c r="H82" s="11" t="s">
-        <v>1106</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22390,7 +22431,7 @@
         <v>1062</v>
       </c>
       <c r="D83" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E83" s="11"/>
       <c r="F83" s="11" t="n">
@@ -22398,7 +22439,7 @@
       </c>
       <c r="G83" s="11"/>
       <c r="H83" s="11" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22406,7 +22447,7 @@
         <v>95</v>
       </c>
       <c r="B84" s="13" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="C84" s="13" t="s">
         <v>495</v>
@@ -22432,7 +22473,7 @@
         <v>1062</v>
       </c>
       <c r="D85" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E85" s="11"/>
       <c r="F85" s="11" t="n">
@@ -22440,7 +22481,7 @@
       </c>
       <c r="G85" s="11"/>
       <c r="H85" s="11" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22454,7 +22495,7 @@
         <v>1062</v>
       </c>
       <c r="D86" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E86" s="11"/>
       <c r="F86" s="11" t="n">
@@ -22462,7 +22503,7 @@
       </c>
       <c r="G86" s="11"/>
       <c r="H86" s="11" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22470,13 +22511,13 @@
         <v>95</v>
       </c>
       <c r="B87" s="11" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="C87" s="11" t="s">
         <v>1062</v>
       </c>
       <c r="D87" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E87" s="11"/>
       <c r="F87" s="11" t="n">
@@ -22484,7 +22525,7 @@
       </c>
       <c r="G87" s="11"/>
       <c r="H87" s="11" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22498,7 +22539,7 @@
         <v>1062</v>
       </c>
       <c r="D88" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E88" s="11"/>
       <c r="F88" s="11" t="n">
@@ -22506,7 +22547,7 @@
       </c>
       <c r="G88" s="11"/>
       <c r="H88" s="11" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22520,7 +22561,7 @@
         <v>1062</v>
       </c>
       <c r="D89" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E89" s="11"/>
       <c r="F89" s="11" t="n">
@@ -22528,7 +22569,7 @@
       </c>
       <c r="G89" s="11"/>
       <c r="H89" s="11" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22542,7 +22583,7 @@
         <v>1062</v>
       </c>
       <c r="D90" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E90" s="11"/>
       <c r="F90" s="11" t="n">
@@ -22550,7 +22591,7 @@
       </c>
       <c r="G90" s="11"/>
       <c r="H90" s="11" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22564,7 +22605,7 @@
         <v>1062</v>
       </c>
       <c r="D91" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E91" s="11"/>
       <c r="F91" s="11" t="n">
@@ -22572,7 +22613,7 @@
       </c>
       <c r="G91" s="11"/>
       <c r="H91" s="11" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22586,17 +22627,17 @@
         <v>1062</v>
       </c>
       <c r="D92" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E92" s="11"/>
       <c r="F92" s="11" t="n">
         <v>1</v>
       </c>
       <c r="G92" s="11" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="H92" s="11" t="s">
-        <v>1118</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22610,7 +22651,7 @@
         <v>1062</v>
       </c>
       <c r="D93" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E93" s="11"/>
       <c r="F93" s="11" t="n">
@@ -22618,7 +22659,7 @@
       </c>
       <c r="G93" s="11"/>
       <c r="H93" s="11" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22632,7 +22673,7 @@
         <v>1062</v>
       </c>
       <c r="D94" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E94" s="11"/>
       <c r="F94" s="11" t="n">
@@ -22640,7 +22681,7 @@
       </c>
       <c r="G94" s="11"/>
       <c r="H94" s="11" t="s">
-        <v>1120</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22654,7 +22695,7 @@
         <v>1062</v>
       </c>
       <c r="D95" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E95" s="11"/>
       <c r="F95" s="11" t="n">
@@ -22662,7 +22703,7 @@
       </c>
       <c r="G95" s="11"/>
       <c r="H95" s="11" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22676,7 +22717,7 @@
         <v>1062</v>
       </c>
       <c r="D96" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E96" s="11"/>
       <c r="F96" s="11" t="n">
@@ -22684,7 +22725,7 @@
       </c>
       <c r="G96" s="11"/>
       <c r="H96" s="11" t="s">
-        <v>1122</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22698,7 +22739,7 @@
         <v>1062</v>
       </c>
       <c r="D97" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E97" s="11"/>
       <c r="F97" s="11" t="n">
@@ -22706,7 +22747,7 @@
       </c>
       <c r="G97" s="11"/>
       <c r="H97" s="11" t="s">
-        <v>1123</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22720,7 +22761,7 @@
         <v>1062</v>
       </c>
       <c r="D98" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E98" s="11"/>
       <c r="F98" s="11" t="n">
@@ -22728,7 +22769,7 @@
       </c>
       <c r="G98" s="11"/>
       <c r="H98" s="11" t="s">
-        <v>1124</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22742,7 +22783,7 @@
         <v>1062</v>
       </c>
       <c r="D99" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E99" s="11"/>
       <c r="F99" s="11" t="n">
@@ -22750,7 +22791,7 @@
       </c>
       <c r="G99" s="11"/>
       <c r="H99" s="11" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22764,7 +22805,7 @@
         <v>1062</v>
       </c>
       <c r="D100" s="11" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="E100" s="11"/>
       <c r="F100" s="11" t="n">
@@ -22772,7 +22813,7 @@
       </c>
       <c r="G100" s="11"/>
       <c r="H100" s="11" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22840,7 +22881,7 @@
         <v>95</v>
       </c>
       <c r="B104" s="13" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="C104" s="13" t="s">
         <v>495</v>
@@ -22860,7 +22901,7 @@
         <v>95</v>
       </c>
       <c r="B105" s="13" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="C105" s="13" t="s">
         <v>495</v>
@@ -22893,7 +22934,7 @@
         <v>1</v>
       </c>
       <c r="G106" s="11" t="s">
-        <v>1129</v>
+        <v>1130</v>
       </c>
       <c r="H106" s="11" t="s">
         <v>1080</v>
@@ -22907,17 +22948,17 @@
         <v>121</v>
       </c>
       <c r="C107" s="11" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="D107" s="11" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="E107" s="11"/>
       <c r="F107" s="11" t="n">
         <v>1</v>
       </c>
       <c r="G107" s="11" t="s">
-        <v>1130</v>
+        <v>1131</v>
       </c>
       <c r="H107" s="11" t="s">
         <v>1080</v>
@@ -22941,7 +22982,7 @@
         <v>1</v>
       </c>
       <c r="G108" s="11" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="H108" s="11" t="s">
         <v>1090</v>
@@ -22965,14 +23006,16 @@
         <v>0</v>
       </c>
       <c r="G109" s="13"/>
-      <c r="H109" s="13"/>
+      <c r="H109" s="13" t="s">
+        <v>1133</v>
+      </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="13" t="s">
         <v>95</v>
       </c>
       <c r="B110" s="13" t="s">
-        <v>1132</v>
+        <v>1134</v>
       </c>
       <c r="C110" s="13" t="s">
         <v>322</v>
@@ -23005,7 +23048,7 @@
         <v>1</v>
       </c>
       <c r="G111" s="11" t="s">
-        <v>1133</v>
+        <v>1135</v>
       </c>
       <c r="H111" s="11" t="s">
         <v>1090</v>
@@ -23036,7 +23079,7 @@
         <v>95</v>
       </c>
       <c r="B113" s="13" t="s">
-        <v>1134</v>
+        <v>1136</v>
       </c>
       <c r="C113" s="13" t="s">
         <v>322</v>
@@ -23056,7 +23099,7 @@
         <v>95</v>
       </c>
       <c r="B114" s="13" t="s">
-        <v>1135</v>
+        <v>1137</v>
       </c>
       <c r="C114" s="13" t="s">
         <v>322</v>
@@ -23096,7 +23139,7 @@
         <v>95</v>
       </c>
       <c r="B116" s="13" t="s">
-        <v>1136</v>
+        <v>1138</v>
       </c>
       <c r="C116" s="13" t="s">
         <v>322</v>
@@ -23109,7 +23152,9 @@
         <v>0</v>
       </c>
       <c r="G116" s="13"/>
-      <c r="H116" s="13"/>
+      <c r="H116" s="13" t="s">
+        <v>1139</v>
+      </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="13" t="s">
@@ -23169,7 +23214,7 @@
         <v>1</v>
       </c>
       <c r="G119" s="11" t="s">
-        <v>1137</v>
+        <v>1140</v>
       </c>
       <c r="H119" s="11" t="s">
         <v>1090</v>
@@ -23213,7 +23258,9 @@
         <v>0</v>
       </c>
       <c r="G121" s="13"/>
-      <c r="H121" s="13"/>
+      <c r="H121" s="13" t="s">
+        <v>1141</v>
+      </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="11" t="s">
@@ -23233,7 +23280,7 @@
         <v>1</v>
       </c>
       <c r="G122" s="11" t="s">
-        <v>1138</v>
+        <v>1142</v>
       </c>
       <c r="H122" s="11" t="s">
         <v>1090</v>
@@ -23257,7 +23304,7 @@
         <v>1</v>
       </c>
       <c r="G123" s="11" t="s">
-        <v>1139</v>
+        <v>1143</v>
       </c>
       <c r="H123" s="11" t="s">
         <v>1090</v>
@@ -23281,7 +23328,9 @@
         <v>0</v>
       </c>
       <c r="G124" s="13"/>
-      <c r="H124" s="13"/>
+      <c r="H124" s="13" t="s">
+        <v>1144</v>
+      </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="13" t="s">
@@ -23308,7 +23357,7 @@
         <v>95</v>
       </c>
       <c r="B126" s="13" t="s">
-        <v>1140</v>
+        <v>1145</v>
       </c>
       <c r="C126" s="13" t="s">
         <v>322</v>
@@ -23321,14 +23370,16 @@
         <v>0</v>
       </c>
       <c r="G126" s="13"/>
-      <c r="H126" s="13"/>
+      <c r="H126" s="13" t="s">
+        <v>1146</v>
+      </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="13" t="s">
         <v>95</v>
       </c>
       <c r="B127" s="13" t="s">
-        <v>1141</v>
+        <v>1147</v>
       </c>
       <c r="C127" s="13" t="s">
         <v>322</v>
@@ -23361,7 +23412,7 @@
         <v>1</v>
       </c>
       <c r="G128" s="11" t="s">
-        <v>1142</v>
+        <v>1148</v>
       </c>
       <c r="H128" s="11" t="s">
         <v>1090</v>
@@ -23372,7 +23423,7 @@
         <v>95</v>
       </c>
       <c r="B129" s="13" t="s">
-        <v>1143</v>
+        <v>1149</v>
       </c>
       <c r="C129" s="13" t="s">
         <v>322</v>
@@ -23385,7 +23436,9 @@
         <v>0</v>
       </c>
       <c r="G129" s="13"/>
-      <c r="H129" s="13"/>
+      <c r="H129" s="13" t="s">
+        <v>1150</v>
+      </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="13" t="s">
@@ -23401,7 +23454,7 @@
         <v>317</v>
       </c>
       <c r="E130" s="13" t="s">
-        <v>1144</v>
+        <v>1151</v>
       </c>
       <c r="F130" s="13" t="n">
         <v>0</v>
@@ -23427,7 +23480,7 @@
         <v>1</v>
       </c>
       <c r="G131" s="11" t="s">
-        <v>1145</v>
+        <v>1152</v>
       </c>
       <c r="H131" s="11" t="s">
         <v>1090</v>
@@ -23451,7 +23504,9 @@
         <v>0</v>
       </c>
       <c r="G132" s="13"/>
-      <c r="H132" s="13"/>
+      <c r="H132" s="13" t="s">
+        <v>1153</v>
+      </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="13" t="s">
@@ -23491,7 +23546,9 @@
         <v>0</v>
       </c>
       <c r="G134" s="13"/>
-      <c r="H134" s="13"/>
+      <c r="H134" s="13" t="s">
+        <v>1154</v>
+      </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="11" t="s">
@@ -23511,7 +23568,7 @@
         <v>1</v>
       </c>
       <c r="G135" s="11" t="s">
-        <v>1146</v>
+        <v>1155</v>
       </c>
       <c r="H135" s="11" t="s">
         <v>1090</v>
@@ -23535,7 +23592,9 @@
         <v>0</v>
       </c>
       <c r="G136" s="13"/>
-      <c r="H136" s="13"/>
+      <c r="H136" s="13" t="s">
+        <v>1156</v>
+      </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="13" t="s">
@@ -23575,7 +23634,9 @@
         <v>0</v>
       </c>
       <c r="G138" s="13"/>
-      <c r="H138" s="13"/>
+      <c r="H138" s="13" t="s">
+        <v>1157</v>
+      </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="17" t="s">
@@ -23595,7 +23656,7 @@
         <v>1</v>
       </c>
       <c r="G139" s="17" t="s">
-        <v>1147</v>
+        <v>1158</v>
       </c>
       <c r="H139" s="17"/>
     </row>
@@ -23677,7 +23738,7 @@
         <v>1</v>
       </c>
       <c r="G143" s="11" t="s">
-        <v>1148</v>
+        <v>1159</v>
       </c>
       <c r="H143" s="11" t="s">
         <v>1090</v>
@@ -23708,7 +23769,7 @@
         <v>135</v>
       </c>
       <c r="B145" s="13" t="s">
-        <v>1149</v>
+        <v>1160</v>
       </c>
       <c r="C145" s="13" t="s">
         <v>495</v>
@@ -23761,7 +23822,7 @@
         <v>1</v>
       </c>
       <c r="G147" s="11" t="s">
-        <v>1150</v>
+        <v>1161</v>
       </c>
       <c r="H147" s="11" t="s">
         <v>1080</v>
@@ -23772,7 +23833,7 @@
         <v>135</v>
       </c>
       <c r="B148" s="13" t="s">
-        <v>1151</v>
+        <v>1162</v>
       </c>
       <c r="C148" s="13" t="s">
         <v>495</v>
@@ -23892,7 +23953,7 @@
         <v>135</v>
       </c>
       <c r="B154" s="13" t="s">
-        <v>1152</v>
+        <v>1163</v>
       </c>
       <c r="C154" s="13" t="s">
         <v>495</v>
@@ -23912,7 +23973,7 @@
         <v>135</v>
       </c>
       <c r="B155" s="13" t="s">
-        <v>1153</v>
+        <v>1164</v>
       </c>
       <c r="C155" s="13" t="s">
         <v>495</v>
@@ -23965,7 +24026,7 @@
         <v>1</v>
       </c>
       <c r="G157" s="11" t="s">
-        <v>1154</v>
+        <v>1165</v>
       </c>
       <c r="H157" s="11" t="s">
         <v>1080</v>
@@ -24196,7 +24257,7 @@
         <v>135</v>
       </c>
       <c r="B169" s="13" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="C169" s="13" t="s">
         <v>322</v>
@@ -24229,7 +24290,9 @@
         <v>0</v>
       </c>
       <c r="G170" s="13"/>
-      <c r="H170" s="13"/>
+      <c r="H170" s="13" t="s">
+        <v>1166</v>
+      </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="11" t="s">
@@ -24249,7 +24312,7 @@
         <v>1</v>
       </c>
       <c r="G171" s="11" t="s">
-        <v>1155</v>
+        <v>1167</v>
       </c>
       <c r="H171" s="11" t="s">
         <v>1090</v>
@@ -24260,7 +24323,7 @@
         <v>135</v>
       </c>
       <c r="B172" s="13" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="C172" s="13" t="s">
         <v>322</v>
@@ -24343,7 +24406,7 @@
         <v>149</v>
       </c>
       <c r="C176" s="17" t="s">
-        <v>1156</v>
+        <v>1168</v>
       </c>
       <c r="D176" s="17" t="s">
         <v>323</v>
@@ -24353,7 +24416,7 @@
         <v>1</v>
       </c>
       <c r="G176" s="17" t="s">
-        <v>1157</v>
+        <v>1169</v>
       </c>
       <c r="H176" s="17"/>
     </row>
@@ -24362,7 +24425,7 @@
         <v>135</v>
       </c>
       <c r="B177" s="13" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="C177" s="13" t="s">
         <v>322</v>
@@ -24375,14 +24438,16 @@
         <v>0</v>
       </c>
       <c r="G177" s="13"/>
-      <c r="H177" s="13"/>
+      <c r="H177" s="13" t="s">
+        <v>1170</v>
+      </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="13" t="s">
         <v>135</v>
       </c>
       <c r="B178" s="13" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="C178" s="13" t="s">
         <v>322</v>
@@ -24455,7 +24520,7 @@
         <v>1</v>
       </c>
       <c r="G181" s="17" t="s">
-        <v>1158</v>
+        <v>1171</v>
       </c>
       <c r="H181" s="17"/>
     </row>
@@ -24464,7 +24529,7 @@
         <v>135</v>
       </c>
       <c r="B182" s="13" t="s">
-        <v>1159</v>
+        <v>1172</v>
       </c>
       <c r="C182" s="13" t="s">
         <v>322</v>
@@ -24484,10 +24549,10 @@
         <v>135</v>
       </c>
       <c r="B183" s="13" t="s">
-        <v>1160</v>
+        <v>1173</v>
       </c>
       <c r="C183" s="13" t="s">
-        <v>1156</v>
+        <v>1168</v>
       </c>
       <c r="D183" s="13" t="s">
         <v>323</v>
@@ -24504,7 +24569,7 @@
         <v>135</v>
       </c>
       <c r="B184" s="13" t="s">
-        <v>1161</v>
+        <v>1174</v>
       </c>
       <c r="C184" s="13" t="s">
         <v>322</v>
@@ -24524,7 +24589,7 @@
         <v>135</v>
       </c>
       <c r="B185" s="13" t="s">
-        <v>1162</v>
+        <v>1175</v>
       </c>
       <c r="C185" s="13" t="s">
         <v>322</v>
@@ -24604,7 +24669,7 @@
         <v>135</v>
       </c>
       <c r="B189" s="13" t="s">
-        <v>1134</v>
+        <v>1136</v>
       </c>
       <c r="C189" s="13" t="s">
         <v>322</v>
@@ -24637,7 +24702,7 @@
         <v>1</v>
       </c>
       <c r="G190" s="11" t="s">
-        <v>1163</v>
+        <v>1176</v>
       </c>
       <c r="H190" s="11" t="s">
         <v>1090</v>
@@ -24661,7 +24726,7 @@
         <v>1</v>
       </c>
       <c r="G191" s="11" t="s">
-        <v>1164</v>
+        <v>1177</v>
       </c>
       <c r="H191" s="11" t="s">
         <v>1090</v>
@@ -24715,7 +24780,7 @@
         <v>532</v>
       </c>
       <c r="C194" s="13" t="s">
-        <v>1156</v>
+        <v>1168</v>
       </c>
       <c r="D194" s="13" t="s">
         <v>323</v>
@@ -24745,7 +24810,7 @@
         <v>1</v>
       </c>
       <c r="G195" s="11" t="s">
-        <v>1165</v>
+        <v>1178</v>
       </c>
       <c r="H195" s="11" t="s">
         <v>1090</v>
@@ -24809,7 +24874,7 @@
         <v>1</v>
       </c>
       <c r="G198" s="11" t="s">
-        <v>1166</v>
+        <v>1179</v>
       </c>
       <c r="H198" s="11" t="s">
         <v>1090</v>
@@ -24860,7 +24925,7 @@
         <v>135</v>
       </c>
       <c r="B201" s="13" t="s">
-        <v>1140</v>
+        <v>1145</v>
       </c>
       <c r="C201" s="13" t="s">
         <v>322</v>
@@ -24880,7 +24945,7 @@
         <v>135</v>
       </c>
       <c r="B202" s="13" t="s">
-        <v>1141</v>
+        <v>1147</v>
       </c>
       <c r="C202" s="13" t="s">
         <v>322</v>
@@ -24900,7 +24965,7 @@
         <v>135</v>
       </c>
       <c r="B203" s="13" t="s">
-        <v>1143</v>
+        <v>1149</v>
       </c>
       <c r="C203" s="13" t="s">
         <v>322</v>
@@ -24929,7 +24994,7 @@
         <v>1062</v>
       </c>
       <c r="E204" s="13" t="s">
-        <v>1167</v>
+        <v>1180</v>
       </c>
       <c r="F204" s="13" t="n">
         <v>0</v>
@@ -24951,7 +25016,7 @@
         <v>1062</v>
       </c>
       <c r="E205" s="13" t="s">
-        <v>1167</v>
+        <v>1180</v>
       </c>
       <c r="F205" s="13" t="n">
         <v>0</v>
@@ -24973,7 +25038,7 @@
         <v>1064</v>
       </c>
       <c r="E206" s="16" t="s">
-        <v>1168</v>
+        <v>1181</v>
       </c>
       <c r="F206" s="16" t="n">
         <v>0</v>
@@ -24997,7 +25062,7 @@
         <v>1062</v>
       </c>
       <c r="E207" s="13" t="s">
-        <v>1167</v>
+        <v>1180</v>
       </c>
       <c r="F207" s="13" t="n">
         <v>0</v>
@@ -25019,7 +25084,7 @@
         <v>1062</v>
       </c>
       <c r="E208" s="13" t="s">
-        <v>1167</v>
+        <v>1180</v>
       </c>
       <c r="F208" s="13" t="n">
         <v>0</v>
@@ -25041,7 +25106,7 @@
         <v>1064</v>
       </c>
       <c r="E209" s="16" t="s">
-        <v>1167</v>
+        <v>1180</v>
       </c>
       <c r="F209" s="16" t="n">
         <v>0</v>
@@ -25065,7 +25130,7 @@
         <v>1062</v>
       </c>
       <c r="E210" s="13" t="s">
-        <v>1167</v>
+        <v>1180</v>
       </c>
       <c r="F210" s="13" t="n">
         <v>0</v>
@@ -25087,7 +25152,7 @@
         <v>1062</v>
       </c>
       <c r="E211" s="13" t="s">
-        <v>1169</v>
+        <v>1182</v>
       </c>
       <c r="F211" s="13" t="n">
         <v>0</v>
@@ -25109,7 +25174,7 @@
         <v>1062</v>
       </c>
       <c r="E212" s="13" t="s">
-        <v>1169</v>
+        <v>1182</v>
       </c>
       <c r="F212" s="13" t="n">
         <v>0</v>
@@ -25131,7 +25196,7 @@
         <v>1062</v>
       </c>
       <c r="E213" s="13" t="s">
-        <v>1169</v>
+        <v>1182</v>
       </c>
       <c r="F213" s="13" t="n">
         <v>0</v>
@@ -25153,13 +25218,13 @@
         <v>1062</v>
       </c>
       <c r="E214" s="11" t="s">
-        <v>1169</v>
+        <v>1182</v>
       </c>
       <c r="F214" s="11" t="n">
         <v>1</v>
       </c>
       <c r="G214" s="11" t="s">
-        <v>1170</v>
+        <v>1183</v>
       </c>
       <c r="H214" s="11" t="s">
         <v>1080</v>
@@ -25179,7 +25244,7 @@
         <v>1062</v>
       </c>
       <c r="E215" s="13" t="s">
-        <v>1169</v>
+        <v>1182</v>
       </c>
       <c r="F215" s="13" t="n">
         <v>0</v>
@@ -25201,7 +25266,7 @@
         <v>1062</v>
       </c>
       <c r="E216" s="13" t="s">
-        <v>1169</v>
+        <v>1182</v>
       </c>
       <c r="F216" s="13" t="n">
         <v>0</v>
@@ -25223,7 +25288,7 @@
         <v>1062</v>
       </c>
       <c r="E217" s="13" t="s">
-        <v>1169</v>
+        <v>1182</v>
       </c>
       <c r="F217" s="13" t="n">
         <v>0</v>
@@ -25267,7 +25332,7 @@
         <v>1062</v>
       </c>
       <c r="E219" s="13" t="s">
-        <v>1169</v>
+        <v>1182</v>
       </c>
       <c r="F219" s="13" t="n">
         <v>0</v>
@@ -25289,7 +25354,7 @@
         <v>1062</v>
       </c>
       <c r="E220" s="13" t="s">
-        <v>1169</v>
+        <v>1182</v>
       </c>
       <c r="F220" s="13" t="n">
         <v>0</v>
@@ -25311,7 +25376,7 @@
         <v>1062</v>
       </c>
       <c r="E221" s="13" t="s">
-        <v>1169</v>
+        <v>1182</v>
       </c>
       <c r="F221" s="13" t="n">
         <v>0</v>
@@ -25333,7 +25398,7 @@
         <v>1062</v>
       </c>
       <c r="E222" s="13" t="s">
-        <v>1169</v>
+        <v>1182</v>
       </c>
       <c r="F222" s="13" t="n">
         <v>0</v>
@@ -25355,7 +25420,7 @@
         <v>1062</v>
       </c>
       <c r="E223" s="13" t="s">
-        <v>1169</v>
+        <v>1182</v>
       </c>
       <c r="F223" s="13" t="n">
         <v>0</v>
@@ -25368,7 +25433,7 @@
         <v>59</v>
       </c>
       <c r="B224" s="13" t="s">
-        <v>1171</v>
+        <v>1184</v>
       </c>
       <c r="C224" s="13" t="s">
         <v>495</v>
@@ -25377,7 +25442,7 @@
         <v>1062</v>
       </c>
       <c r="E224" s="13" t="s">
-        <v>1172</v>
+        <v>1185</v>
       </c>
       <c r="F224" s="13" t="n">
         <v>0</v>
@@ -25390,7 +25455,7 @@
         <v>59</v>
       </c>
       <c r="B225" s="13" t="s">
-        <v>1173</v>
+        <v>1186</v>
       </c>
       <c r="C225" s="13" t="s">
         <v>495</v>
@@ -25399,7 +25464,7 @@
         <v>1062</v>
       </c>
       <c r="E225" s="13" t="s">
-        <v>1169</v>
+        <v>1182</v>
       </c>
       <c r="F225" s="13" t="n">
         <v>0</v>
@@ -25412,7 +25477,7 @@
         <v>59</v>
       </c>
       <c r="B226" s="13" t="s">
-        <v>1174</v>
+        <v>1187</v>
       </c>
       <c r="C226" s="13" t="s">
         <v>495</v>
@@ -25421,7 +25486,7 @@
         <v>1062</v>
       </c>
       <c r="E226" s="13" t="s">
-        <v>1175</v>
+        <v>1188</v>
       </c>
       <c r="F226" s="13" t="n">
         <v>0</v>
@@ -25554,7 +25619,7 @@
         <v>59</v>
       </c>
       <c r="B233" s="13" t="s">
-        <v>1176</v>
+        <v>1189</v>
       </c>
       <c r="C233" s="13" t="s">
         <v>495</v>
@@ -25574,7 +25639,7 @@
         <v>59</v>
       </c>
       <c r="B234" s="13" t="s">
-        <v>1177</v>
+        <v>1190</v>
       </c>
       <c r="C234" s="13" t="s">
         <v>495</v>
@@ -25594,7 +25659,7 @@
         <v>59</v>
       </c>
       <c r="B235" s="13" t="s">
-        <v>1178</v>
+        <v>1191</v>
       </c>
       <c r="C235" s="13" t="s">
         <v>495</v>
@@ -25614,7 +25679,7 @@
         <v>59</v>
       </c>
       <c r="B236" s="13" t="s">
-        <v>1179</v>
+        <v>1192</v>
       </c>
       <c r="C236" s="13" t="s">
         <v>495</v>
@@ -25663,7 +25728,7 @@
         <v>1064</v>
       </c>
       <c r="E238" s="16" t="s">
-        <v>1168</v>
+        <v>1181</v>
       </c>
       <c r="F238" s="16" t="n">
         <v>0</v>
@@ -25684,7 +25749,7 @@
         <v>317</v>
       </c>
       <c r="D239" s="13" t="s">
-        <v>1180</v>
+        <v>1193</v>
       </c>
       <c r="E239" s="13"/>
       <c r="F239" s="13" t="n">
@@ -25731,7 +25796,7 @@
         <v>1</v>
       </c>
       <c r="G241" s="11" t="s">
-        <v>1181</v>
+        <v>1194</v>
       </c>
       <c r="H241" s="11" t="s">
         <v>1080</v>
@@ -25742,7 +25807,7 @@
         <v>59</v>
       </c>
       <c r="B242" s="13" t="s">
-        <v>1182</v>
+        <v>1195</v>
       </c>
       <c r="C242" s="13" t="s">
         <v>322</v>
@@ -25762,7 +25827,7 @@
         <v>59</v>
       </c>
       <c r="B243" s="13" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="C243" s="13" t="s">
         <v>495</v>
@@ -25782,7 +25847,7 @@
         <v>59</v>
       </c>
       <c r="B244" s="13" t="s">
-        <v>1149</v>
+        <v>1160</v>
       </c>
       <c r="C244" s="13" t="s">
         <v>495</v>
@@ -25822,7 +25887,7 @@
         <v>59</v>
       </c>
       <c r="B246" s="13" t="s">
-        <v>1183</v>
+        <v>1196</v>
       </c>
       <c r="C246" s="13" t="s">
         <v>495</v>
@@ -25862,7 +25927,7 @@
         <v>59</v>
       </c>
       <c r="B248" s="13" t="s">
-        <v>1184</v>
+        <v>1197</v>
       </c>
       <c r="C248" s="13" t="s">
         <v>495</v>
@@ -25882,7 +25947,7 @@
         <v>59</v>
       </c>
       <c r="B249" s="13" t="s">
-        <v>1151</v>
+        <v>1162</v>
       </c>
       <c r="C249" s="13" t="s">
         <v>495</v>
@@ -25902,7 +25967,7 @@
         <v>59</v>
       </c>
       <c r="B250" s="13" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="C250" s="13" t="s">
         <v>495</v>
@@ -25922,7 +25987,7 @@
         <v>59</v>
       </c>
       <c r="B251" s="13" t="s">
-        <v>1152</v>
+        <v>1163</v>
       </c>
       <c r="C251" s="13" t="s">
         <v>495</v>
@@ -25942,7 +26007,7 @@
         <v>59</v>
       </c>
       <c r="B252" s="13" t="s">
-        <v>1153</v>
+        <v>1164</v>
       </c>
       <c r="C252" s="13" t="s">
         <v>495</v>
@@ -25962,7 +26027,7 @@
         <v>59</v>
       </c>
       <c r="B253" s="13" t="s">
-        <v>1185</v>
+        <v>1198</v>
       </c>
       <c r="C253" s="13" t="s">
         <v>495</v>
@@ -25995,7 +26060,7 @@
         <v>1</v>
       </c>
       <c r="G254" s="11" t="s">
-        <v>1186</v>
+        <v>1199</v>
       </c>
       <c r="H254" s="11" t="s">
         <v>1080</v>
@@ -26006,7 +26071,7 @@
         <v>59</v>
       </c>
       <c r="B255" s="13" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="C255" s="13" t="s">
         <v>495</v>
@@ -26046,7 +26111,7 @@
         <v>59</v>
       </c>
       <c r="B257" s="13" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="C257" s="13" t="s">
         <v>495</v>
@@ -26146,7 +26211,7 @@
         <v>59</v>
       </c>
       <c r="B262" s="13" t="s">
-        <v>1134</v>
+        <v>1136</v>
       </c>
       <c r="C262" s="13" t="s">
         <v>495</v>
@@ -26166,7 +26231,7 @@
         <v>59</v>
       </c>
       <c r="B263" s="13" t="s">
-        <v>1135</v>
+        <v>1137</v>
       </c>
       <c r="C263" s="13" t="s">
         <v>495</v>
@@ -26266,7 +26331,7 @@
         <v>59</v>
       </c>
       <c r="B268" s="13" t="s">
-        <v>1136</v>
+        <v>1138</v>
       </c>
       <c r="C268" s="13" t="s">
         <v>495</v>
@@ -26659,7 +26724,7 @@
         <v>1</v>
       </c>
       <c r="G287" s="11" t="s">
-        <v>1187</v>
+        <v>1200</v>
       </c>
       <c r="H287" s="11" t="s">
         <v>1080</v>
@@ -26739,7 +26804,7 @@
         <v>317</v>
       </c>
       <c r="E291" s="13" t="s">
-        <v>1188</v>
+        <v>1201</v>
       </c>
       <c r="F291" s="13" t="n">
         <v>0</v>
@@ -26812,7 +26877,7 @@
         <v>59</v>
       </c>
       <c r="B295" s="13" t="s">
-        <v>1140</v>
+        <v>1145</v>
       </c>
       <c r="C295" s="13" t="s">
         <v>495</v>
@@ -26852,7 +26917,7 @@
         <v>59</v>
       </c>
       <c r="B297" s="13" t="s">
-        <v>1141</v>
+        <v>1147</v>
       </c>
       <c r="C297" s="13" t="s">
         <v>495</v>
@@ -26932,7 +26997,7 @@
         <v>59</v>
       </c>
       <c r="B301" s="13" t="s">
-        <v>1143</v>
+        <v>1149</v>
       </c>
       <c r="C301" s="13" t="s">
         <v>495</v>
@@ -26965,7 +27030,7 @@
         <v>1</v>
       </c>
       <c r="G302" s="11" t="s">
-        <v>1189</v>
+        <v>1202</v>
       </c>
       <c r="H302" s="11" t="s">
         <v>1080</v>
@@ -26976,7 +27041,7 @@
         <v>59</v>
       </c>
       <c r="B303" s="13" t="s">
-        <v>1190</v>
+        <v>1203</v>
       </c>
       <c r="C303" s="13" t="s">
         <v>495</v>
@@ -26996,7 +27061,7 @@
         <v>59</v>
       </c>
       <c r="B304" s="13" t="s">
-        <v>1191</v>
+        <v>1204</v>
       </c>
       <c r="C304" s="13" t="s">
         <v>495</v>
@@ -27016,7 +27081,7 @@
         <v>59</v>
       </c>
       <c r="B305" s="13" t="s">
-        <v>1192</v>
+        <v>1205</v>
       </c>
       <c r="C305" s="13" t="s">
         <v>495</v>
@@ -27036,7 +27101,7 @@
         <v>59</v>
       </c>
       <c r="B306" s="13" t="s">
-        <v>1193</v>
+        <v>1206</v>
       </c>
       <c r="C306" s="13" t="s">
         <v>495</v>
@@ -27056,7 +27121,7 @@
         <v>59</v>
       </c>
       <c r="B307" s="13" t="s">
-        <v>1194</v>
+        <v>1207</v>
       </c>
       <c r="C307" s="13" t="s">
         <v>495</v>
@@ -27076,7 +27141,7 @@
         <v>59</v>
       </c>
       <c r="B308" s="13" t="s">
-        <v>1195</v>
+        <v>1208</v>
       </c>
       <c r="C308" s="13" t="s">
         <v>495</v>
@@ -27096,7 +27161,7 @@
         <v>59</v>
       </c>
       <c r="B309" s="13" t="s">
-        <v>1196</v>
+        <v>1209</v>
       </c>
       <c r="C309" s="13" t="s">
         <v>495</v>
@@ -27116,7 +27181,7 @@
         <v>59</v>
       </c>
       <c r="B310" s="13" t="s">
-        <v>1197</v>
+        <v>1210</v>
       </c>
       <c r="C310" s="13" t="s">
         <v>495</v>
@@ -27136,7 +27201,7 @@
         <v>59</v>
       </c>
       <c r="B311" s="13" t="s">
-        <v>1198</v>
+        <v>1211</v>
       </c>
       <c r="C311" s="13" t="s">
         <v>495</v>
@@ -27156,7 +27221,7 @@
         <v>59</v>
       </c>
       <c r="B312" s="13" t="s">
-        <v>1199</v>
+        <v>1212</v>
       </c>
       <c r="C312" s="13" t="s">
         <v>495</v>
@@ -27176,7 +27241,7 @@
         <v>59</v>
       </c>
       <c r="B313" s="13" t="s">
-        <v>1200</v>
+        <v>1213</v>
       </c>
       <c r="C313" s="13" t="s">
         <v>495</v>
@@ -27196,7 +27261,7 @@
         <v>59</v>
       </c>
       <c r="B314" s="13" t="s">
-        <v>1201</v>
+        <v>1214</v>
       </c>
       <c r="C314" s="13" t="s">
         <v>495</v>
@@ -27216,7 +27281,7 @@
         <v>59</v>
       </c>
       <c r="B315" s="13" t="s">
-        <v>1202</v>
+        <v>1215</v>
       </c>
       <c r="C315" s="13" t="s">
         <v>495</v>
@@ -27236,7 +27301,7 @@
         <v>59</v>
       </c>
       <c r="B316" s="13" t="s">
-        <v>1203</v>
+        <v>1216</v>
       </c>
       <c r="C316" s="13" t="s">
         <v>495</v>
@@ -27256,7 +27321,7 @@
         <v>59</v>
       </c>
       <c r="B317" s="13" t="s">
-        <v>1204</v>
+        <v>1217</v>
       </c>
       <c r="C317" s="13" t="s">
         <v>495</v>
@@ -27289,7 +27354,7 @@
         <v>1</v>
       </c>
       <c r="G318" s="11" t="s">
-        <v>1205</v>
+        <v>1218</v>
       </c>
       <c r="H318" s="11" t="s">
         <v>1080</v>
@@ -27300,7 +27365,7 @@
         <v>59</v>
       </c>
       <c r="B319" s="13" t="s">
-        <v>1206</v>
+        <v>1219</v>
       </c>
       <c r="C319" s="13" t="s">
         <v>495</v>
@@ -27320,7 +27385,7 @@
         <v>59</v>
       </c>
       <c r="B320" s="13" t="s">
-        <v>1207</v>
+        <v>1220</v>
       </c>
       <c r="C320" s="13" t="s">
         <v>495</v>
@@ -27340,7 +27405,7 @@
         <v>59</v>
       </c>
       <c r="B321" s="13" t="s">
-        <v>1208</v>
+        <v>1221</v>
       </c>
       <c r="C321" s="13" t="s">
         <v>322</v>
@@ -27360,7 +27425,7 @@
         <v>59</v>
       </c>
       <c r="B322" s="13" t="s">
-        <v>1209</v>
+        <v>1222</v>
       </c>
       <c r="C322" s="13" t="s">
         <v>495</v>
@@ -27393,7 +27458,7 @@
         <v>1</v>
       </c>
       <c r="G323" s="11" t="s">
-        <v>1210</v>
+        <v>1223</v>
       </c>
       <c r="H323" s="11" t="s">
         <v>1080</v>
@@ -27404,7 +27469,7 @@
         <v>59</v>
       </c>
       <c r="B324" s="13" t="s">
-        <v>1211</v>
+        <v>1224</v>
       </c>
       <c r="C324" s="13" t="s">
         <v>322</v>
@@ -27424,7 +27489,7 @@
         <v>59</v>
       </c>
       <c r="B325" s="13" t="s">
-        <v>1212</v>
+        <v>1225</v>
       </c>
       <c r="C325" s="13" t="s">
         <v>495</v>
@@ -27444,7 +27509,7 @@
         <v>59</v>
       </c>
       <c r="B326" s="13" t="s">
-        <v>1213</v>
+        <v>1226</v>
       </c>
       <c r="C326" s="13" t="s">
         <v>322</v>
@@ -27464,7 +27529,7 @@
         <v>59</v>
       </c>
       <c r="B327" s="13" t="s">
-        <v>1214</v>
+        <v>1227</v>
       </c>
       <c r="C327" s="13" t="s">
         <v>495</v>
@@ -27497,7 +27562,7 @@
         <v>1</v>
       </c>
       <c r="G328" s="11" t="s">
-        <v>1215</v>
+        <v>1228</v>
       </c>
       <c r="H328" s="11" t="s">
         <v>1080</v>
@@ -27508,7 +27573,7 @@
         <v>59</v>
       </c>
       <c r="B329" s="13" t="s">
-        <v>1216</v>
+        <v>1229</v>
       </c>
       <c r="C329" s="13" t="s">
         <v>495</v>
@@ -27528,7 +27593,7 @@
         <v>59</v>
       </c>
       <c r="B330" s="13" t="s">
-        <v>1217</v>
+        <v>1230</v>
       </c>
       <c r="C330" s="13" t="s">
         <v>495</v>
@@ -27548,7 +27613,7 @@
         <v>59</v>
       </c>
       <c r="B331" s="13" t="s">
-        <v>1218</v>
+        <v>1231</v>
       </c>
       <c r="C331" s="13" t="s">
         <v>495</v>
@@ -27568,7 +27633,7 @@
         <v>59</v>
       </c>
       <c r="B332" s="13" t="s">
-        <v>1219</v>
+        <v>1232</v>
       </c>
       <c r="C332" s="13" t="s">
         <v>495</v>
@@ -27588,7 +27653,7 @@
         <v>59</v>
       </c>
       <c r="B333" s="13" t="s">
-        <v>1220</v>
+        <v>1233</v>
       </c>
       <c r="C333" s="13" t="s">
         <v>495</v>
@@ -27608,7 +27673,7 @@
         <v>59</v>
       </c>
       <c r="B334" s="13" t="s">
-        <v>1221</v>
+        <v>1234</v>
       </c>
       <c r="C334" s="13" t="s">
         <v>495</v>
@@ -27628,7 +27693,7 @@
         <v>59</v>
       </c>
       <c r="B335" s="13" t="s">
-        <v>1222</v>
+        <v>1235</v>
       </c>
       <c r="C335" s="13" t="s">
         <v>495</v>
@@ -27648,7 +27713,7 @@
         <v>59</v>
       </c>
       <c r="B336" s="13" t="s">
-        <v>1223</v>
+        <v>1236</v>
       </c>
       <c r="C336" s="13" t="s">
         <v>495</v>
@@ -27668,7 +27733,7 @@
         <v>59</v>
       </c>
       <c r="B337" s="13" t="s">
-        <v>1224</v>
+        <v>1237</v>
       </c>
       <c r="C337" s="13" t="s">
         <v>495</v>
@@ -27697,7 +27762,7 @@
         <v>1064</v>
       </c>
       <c r="E338" s="16" t="s">
-        <v>1168</v>
+        <v>1181</v>
       </c>
       <c r="F338" s="16" t="n">
         <v>0</v>
@@ -27712,7 +27777,7 @@
         <v>59</v>
       </c>
       <c r="B339" s="13" t="s">
-        <v>1225</v>
+        <v>1238</v>
       </c>
       <c r="C339" s="13" t="s">
         <v>495</v>
@@ -27732,7 +27797,7 @@
         <v>59</v>
       </c>
       <c r="B340" s="13" t="s">
-        <v>1226</v>
+        <v>1239</v>
       </c>
       <c r="C340" s="13" t="s">
         <v>495</v>
@@ -27752,7 +27817,7 @@
         <v>59</v>
       </c>
       <c r="B341" s="13" t="s">
-        <v>1227</v>
+        <v>1240</v>
       </c>
       <c r="C341" s="13" t="s">
         <v>322</v>
@@ -27772,7 +27837,7 @@
         <v>59</v>
       </c>
       <c r="B342" s="13" t="s">
-        <v>1228</v>
+        <v>1241</v>
       </c>
       <c r="C342" s="13" t="s">
         <v>495</v>
@@ -27792,7 +27857,7 @@
         <v>59</v>
       </c>
       <c r="B343" s="13" t="s">
-        <v>1229</v>
+        <v>1242</v>
       </c>
       <c r="C343" s="13" t="s">
         <v>495</v>
@@ -27812,7 +27877,7 @@
         <v>59</v>
       </c>
       <c r="B344" s="13" t="s">
-        <v>1230</v>
+        <v>1243</v>
       </c>
       <c r="C344" s="13" t="s">
         <v>495</v>
@@ -27832,7 +27897,7 @@
         <v>59</v>
       </c>
       <c r="B345" s="13" t="s">
-        <v>1231</v>
+        <v>1244</v>
       </c>
       <c r="C345" s="13" t="s">
         <v>495</v>
@@ -27852,7 +27917,7 @@
         <v>59</v>
       </c>
       <c r="B346" s="13" t="s">
-        <v>1232</v>
+        <v>1245</v>
       </c>
       <c r="C346" s="13" t="s">
         <v>495</v>
@@ -27872,7 +27937,7 @@
         <v>59</v>
       </c>
       <c r="B347" s="13" t="s">
-        <v>1233</v>
+        <v>1246</v>
       </c>
       <c r="C347" s="13" t="s">
         <v>495</v>
@@ -27892,7 +27957,7 @@
         <v>59</v>
       </c>
       <c r="B348" s="13" t="s">
-        <v>1234</v>
+        <v>1247</v>
       </c>
       <c r="C348" s="13" t="s">
         <v>495</v>
@@ -27912,7 +27977,7 @@
         <v>59</v>
       </c>
       <c r="B349" s="13" t="s">
-        <v>1235</v>
+        <v>1248</v>
       </c>
       <c r="C349" s="13" t="s">
         <v>495</v>
@@ -27932,7 +27997,7 @@
         <v>59</v>
       </c>
       <c r="B350" s="13" t="s">
-        <v>1236</v>
+        <v>1249</v>
       </c>
       <c r="C350" s="13" t="s">
         <v>495</v>
@@ -27952,7 +28017,7 @@
         <v>59</v>
       </c>
       <c r="B351" s="13" t="s">
-        <v>1237</v>
+        <v>1250</v>
       </c>
       <c r="C351" s="13" t="s">
         <v>495</v>
@@ -27972,7 +28037,7 @@
         <v>59</v>
       </c>
       <c r="B352" s="13" t="s">
-        <v>1238</v>
+        <v>1251</v>
       </c>
       <c r="C352" s="13" t="s">
         <v>495</v>
@@ -27992,7 +28057,7 @@
         <v>59</v>
       </c>
       <c r="B353" s="13" t="s">
-        <v>1239</v>
+        <v>1252</v>
       </c>
       <c r="C353" s="13" t="s">
         <v>495</v>
@@ -28012,7 +28077,7 @@
         <v>59</v>
       </c>
       <c r="B354" s="13" t="s">
-        <v>1240</v>
+        <v>1253</v>
       </c>
       <c r="C354" s="13" t="s">
         <v>495</v>
@@ -28032,7 +28097,7 @@
         <v>59</v>
       </c>
       <c r="B355" s="13" t="s">
-        <v>1241</v>
+        <v>1254</v>
       </c>
       <c r="C355" s="13" t="s">
         <v>495</v>
@@ -28052,7 +28117,7 @@
         <v>59</v>
       </c>
       <c r="B356" s="13" t="s">
-        <v>1242</v>
+        <v>1255</v>
       </c>
       <c r="C356" s="13" t="s">
         <v>495</v>
@@ -28072,7 +28137,7 @@
         <v>59</v>
       </c>
       <c r="B357" s="13" t="s">
-        <v>1243</v>
+        <v>1256</v>
       </c>
       <c r="C357" s="13" t="s">
         <v>495</v>
@@ -28092,7 +28157,7 @@
         <v>59</v>
       </c>
       <c r="B358" s="13" t="s">
-        <v>1244</v>
+        <v>1257</v>
       </c>
       <c r="C358" s="13" t="s">
         <v>322</v>
@@ -28112,7 +28177,7 @@
         <v>59</v>
       </c>
       <c r="B359" s="13" t="s">
-        <v>1245</v>
+        <v>1258</v>
       </c>
       <c r="C359" s="13" t="s">
         <v>322</v>
@@ -28132,7 +28197,7 @@
         <v>59</v>
       </c>
       <c r="B360" s="13" t="s">
-        <v>1246</v>
+        <v>1259</v>
       </c>
       <c r="C360" s="13" t="s">
         <v>495</v>
@@ -28152,7 +28217,7 @@
         <v>59</v>
       </c>
       <c r="B361" s="13" t="s">
-        <v>1247</v>
+        <v>1260</v>
       </c>
       <c r="C361" s="13" t="s">
         <v>495</v>
@@ -28172,7 +28237,7 @@
         <v>59</v>
       </c>
       <c r="B362" s="13" t="s">
-        <v>1248</v>
+        <v>1261</v>
       </c>
       <c r="C362" s="13" t="s">
         <v>495</v>
@@ -28236,7 +28301,7 @@
         <v>310</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>1249</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28247,10 +28312,10 @@
         <v>313</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>1250</v>
+        <v>1263</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>1251</v>
+        <v>1264</v>
       </c>
       <c r="E2" s="13" t="s">
         <v>316</v>
@@ -28259,7 +28324,7 @@
         <v>317</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>1252</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28273,16 +28338,16 @@
         <v>454</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>1253</v>
+        <v>1266</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>1254</v>
+        <v>1267</v>
       </c>
       <c r="F3" s="13" t="s">
         <v>323</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>1252</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28296,16 +28361,16 @@
         <v>454</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>1255</v>
+        <v>1268</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>1254</v>
+        <v>1267</v>
       </c>
       <c r="F4" s="13" t="s">
         <v>323</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>1252</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28319,16 +28384,16 @@
         <v>445</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>1256</v>
+        <v>1269</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>1254</v>
+        <v>1267</v>
       </c>
       <c r="F5" s="13" t="s">
         <v>323</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>1252</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28342,16 +28407,16 @@
         <v>445</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>1257</v>
+        <v>1270</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>1254</v>
+        <v>1267</v>
       </c>
       <c r="F6" s="13" t="s">
         <v>323</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>1252</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28365,16 +28430,16 @@
         <v>445</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>1258</v>
+        <v>1271</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>1254</v>
+        <v>1267</v>
       </c>
       <c r="F7" s="13" t="s">
         <v>323</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>1252</v>
+        <v>1265</v>
       </c>
     </row>
   </sheetData>
@@ -28404,10 +28469,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>1259</v>
+        <v>1272</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>1260</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28416,7 +28481,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>1261</v>
+        <v>1274</v>
       </c>
       <c r="B3" s="18" t="n">
         <f aca="false">COUNTA('200V Devices'!C2:C393)</f>
@@ -28425,7 +28490,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>1262</v>
+        <v>1275</v>
       </c>
       <c r="B4" s="18" t="n">
         <f aca="false">COUNTIF('200V Devices'!I2:I393,"Done (pilot)")</f>
@@ -28434,7 +28499,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>1263</v>
+        <v>1276</v>
       </c>
       <c r="B5" s="18" t="n">
         <f aca="false">COUNTIF('200V Devices'!I2:I393,"Done")</f>
@@ -28443,7 +28508,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>1264</v>
+        <v>1277</v>
       </c>
       <c r="B6" s="18" t="n">
         <f aca="false">COUNTIF('200V Devices'!I2:I393,"To do")</f>
@@ -28452,7 +28517,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>1265</v>
+        <v>1278</v>
       </c>
       <c r="B7" s="18" t="n">
         <f aca="false">COUNTIF('200V Devices'!J2:J393,"Matched from 200V tab")</f>
@@ -28461,7 +28526,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>1266</v>
+        <v>1279</v>
       </c>
       <c r="B8" s="18" t="n">
         <f aca="false">COUNTA('Not found'!C2:C7)</f>
@@ -28470,7 +28535,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>1267</v>
+        <v>1280</v>
       </c>
       <c r="B9" s="18" t="n">
         <f aca="false">B3+B8</f>
@@ -28486,7 +28551,7 @@
         <v>4</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>1268</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28540,30 +28605,30 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
-        <v>1269</v>
+        <v>1282</v>
       </c>
       <c r="B18" s="18"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>1270</v>
+        <v>1283</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>1271</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>1272</v>
+        <v>1285</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>1273</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>1274</v>
+        <v>1287</v>
       </c>
       <c r="B22" s="18" t="n">
         <f aca="false">COUNTA('Ports without device'!A2:A362)</f>
@@ -28572,7 +28637,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>1275</v>
+        <v>1288</v>
       </c>
       <c r="B23" s="18" t="n">
         <f aca="false">COUNTIF('Ports without device'!F2:F362,"&gt;0")</f>
@@ -28581,7 +28646,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>1276</v>
+        <v>1289</v>
       </c>
       <c r="B24" s="18" t="n">
         <f aca="false">COUNTIF('Ports without device'!F2:F362,0)</f>
@@ -28590,7 +28655,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>1277</v>
+        <v>1290</v>
       </c>
       <c r="B25" s="18" t="n">
         <f aca="false">COUNTIF('Ports without device'!H2:H362,"Pilot staff outlet*")</f>
@@ -28599,7 +28664,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>1278</v>
+        <v>1291</v>
       </c>
       <c r="B26" s="18" t="n">
         <f aca="false">COUNTIF('Ports without device'!C2:C362,"None (tagged only)")</f>
@@ -28608,16 +28673,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
-        <v>1279</v>
+        <v>1292</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>1280</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>1281</v>
+        <v>1294</v>
       </c>
       <c r="B29" s="18" t="n">
         <f aca="false">COUNT(Review!A5:A130)</f>
@@ -28626,7 +28691,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="18" t="s">
-        <v>1282</v>
+        <v>1295</v>
       </c>
       <c r="B30" s="18" t="n">
         <f aca="false">COUNTA(Review!H5:H130)</f>
@@ -28635,7 +28700,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="18" t="s">
-        <v>1283</v>
+        <v>1296</v>
       </c>
       <c r="B31" s="18" t="n">
         <f aca="false">B29-B30</f>

</xml_diff>

<commit_message>
Move the 13 20:7B:D2:30 outlets to VLAN 2100 instead of 2700
Replaces 200V-av-207bd2-2700-ICX.txt with 200V-207bd2-2100-ICX.txt and
updates the New VLAN and notes on the Ports without device tab.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZ7jJsE6GWKm6ehHY39VNr
</commit_message>
<xml_diff>
--- a/200V Device Port List.xlsx
+++ b/200V Device Port List.xlsx
@@ -3323,7 +3323,7 @@
     <t xml:space="preserve">Moved to 2700 on 9 Oct (unlisted AV device).</t>
   </si>
   <si>
-    <t xml:space="preserve">AV outlet 200V3J5, device 20:7B:D2:30:98:F3 (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+    <t xml:space="preserve">Outlet 200V3J5, device 20:7B:D2:30:98:F3 (Dycom patching sheet 2025-07-30). To 2100 (decision 9 Oct): 200V-207bd2-2100-ICX.txt.</t>
   </si>
   <si>
     <t xml:space="preserve">D8:43:AE:B1:6E:9B</t>
@@ -3449,7 +3449,7 @@
     <t xml:space="preserve">D8:43:AE:B1:6C:A8</t>
   </si>
   <si>
-    <t xml:space="preserve">AV outlet 200V3G16, device 20:7B:D2:30:98:D6 (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+    <t xml:space="preserve">Outlet 200V3G16, device 20:7B:D2:30:98:D6 (Dycom patching sheet 2025-07-30). To 2100 (decision 9 Oct): 200V-207bd2-2100-ICX.txt.</t>
   </si>
   <si>
     <t xml:space="preserve">4/1/45</t>
@@ -3467,13 +3467,13 @@
     <t xml:space="preserve">5/1/11</t>
   </si>
   <si>
-    <t xml:space="preserve">AV outlet 200V3H2, device 20:7B:D2:30:99:09 (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+    <t xml:space="preserve">Outlet 200V3H2, device 20:7B:D2:30:99:09 (Dycom patching sheet 2025-07-30). To 2100 (decision 9 Oct): 200V-207bd2-2100-ICX.txt.</t>
   </si>
   <si>
     <t xml:space="preserve">D8:43:AE:B1:6E:B0</t>
   </si>
   <si>
-    <t xml:space="preserve">AV outlet 200V3I8, device 20:7B:D2:30:98:AF (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+    <t xml:space="preserve">Outlet 200V3I8, device 20:7B:D2:30:98:AF (Dycom patching sheet 2025-07-30). To 2100 (decision 9 Oct): 200V-207bd2-2100-ICX.txt.</t>
   </si>
   <si>
     <t xml:space="preserve">D8:43:AE:B1:6E:3C</t>
@@ -3482,13 +3482,13 @@
     <t xml:space="preserve">D8:43:AE:B1:6F:04</t>
   </si>
   <si>
-    <t xml:space="preserve">AV outlet 200V3I16, device 20:7B:D2:30:98:D2 (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+    <t xml:space="preserve">Outlet 200V3I16, device 20:7B:D2:30:98:D2 (Dycom patching sheet 2025-07-30). To 2100 (decision 9 Oct): 200V-207bd2-2100-ICX.txt.</t>
   </si>
   <si>
     <t xml:space="preserve">5/1/40</t>
   </si>
   <si>
-    <t xml:space="preserve">AV outlet 200V3H14, device 20:7B:D2:30:98:B1 (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+    <t xml:space="preserve">Outlet 200V3H14, device 20:7B:D2:30:98:B1 (Dycom patching sheet 2025-07-30). To 2100 (decision 9 Oct): 200V-207bd2-2100-ICX.txt.</t>
   </si>
   <si>
     <t xml:space="preserve">5/1/43</t>
@@ -3500,7 +3500,7 @@
     <t xml:space="preserve">5/1/47</t>
   </si>
   <si>
-    <t xml:space="preserve">AV outlet 200V3H21, device 20:7B:D2:30:99:29 (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+    <t xml:space="preserve">Outlet 200V3H21, device 20:7B:D2:30:99:29 (Dycom patching sheet 2025-07-30). To 2100 (decision 9 Oct): 200V-207bd2-2100-ICX.txt.</t>
   </si>
   <si>
     <t xml:space="preserve">1272,1273,2300,2310,2311,2320,2321</t>
@@ -3509,19 +3509,19 @@
     <t xml:space="preserve">D8:43:AE:B1:6E:06</t>
   </si>
   <si>
-    <t xml:space="preserve">AV outlet 200V4H22, device 20:7B:D2:30:98:FD (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AV outlet 200V4I10, device 20:7B:D2:30:98:EF (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+    <t xml:space="preserve">Outlet 200V4H22, device 20:7B:D2:30:98:FD (Dycom patching sheet 2025-07-30). To 2100 (decision 9 Oct): 200V-207bd2-2100-ICX.txt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outlet 200V4I10, device 20:7B:D2:30:98:EF (Dycom patching sheet 2025-07-30). To 2100 (decision 9 Oct): 200V-207bd2-2100-ICX.txt.</t>
   </si>
   <si>
     <t xml:space="preserve">D8:43:AE:B1:6A:29</t>
   </si>
   <si>
-    <t xml:space="preserve">AV outlet 200V4J4, device 20:7B:D2:30:98:DB (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AV outlet 200V4J14, device 20:7B:D2:30:99:0E (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+    <t xml:space="preserve">Outlet 200V4J4, device 20:7B:D2:30:98:DB (Dycom patching sheet 2025-07-30). To 2100 (decision 9 Oct): 200V-207bd2-2100-ICX.txt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outlet 200V4J14, device 20:7B:D2:30:99:0E (Dycom patching sheet 2025-07-30). To 2100 (decision 9 Oct): 200V-207bd2-2100-ICX.txt.</t>
   </si>
   <si>
     <t xml:space="preserve">00:09:F5:32:D9:F7</t>
@@ -3548,7 +3548,7 @@
     <t xml:space="preserve">A0:4A:5E:E7:D5:71</t>
   </si>
   <si>
-    <t xml:space="preserve">AV outlet 200V4F5, device 20:7B:D2:30:98:DF (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+    <t xml:space="preserve">Outlet 200V4F5, device 20:7B:D2:30:98:DF (Dycom patching sheet 2025-07-30). To 2100 (decision 9 Oct): 200V-207bd2-2100-ICX.txt.</t>
   </si>
   <si>
     <t xml:space="preserve">D8:43:AE:B1:6D:56</t>
@@ -3560,7 +3560,7 @@
     <t xml:space="preserve">38:4B:76:E0:B0:B1</t>
   </si>
   <si>
-    <t xml:space="preserve">AV outlet 200V4H2, device 20:7B:D2:30:98:C2 (Dycom patching sheet 2025-07-30). To 2700: 200V-av-207bd2-2700-ICX.txt.</t>
+    <t xml:space="preserve">Outlet 200V4H2, device 20:7B:D2:30:98:C2 (Dycom patching sheet 2025-07-30). To 2100 (decision 9 Oct): 200V-207bd2-2100-ICX.txt.</t>
   </si>
   <si>
     <t xml:space="preserve">F8:25:51:CC:2C:76</t>
@@ -21875,7 +21875,7 @@
         <v>322</v>
       </c>
       <c r="D57" s="13" t="s">
-        <v>323</v>
+        <v>1062</v>
       </c>
       <c r="E57" s="13"/>
       <c r="F57" s="13" t="n">
@@ -22999,7 +22999,7 @@
         <v>322</v>
       </c>
       <c r="D109" s="13" t="s">
-        <v>323</v>
+        <v>1062</v>
       </c>
       <c r="E109" s="13"/>
       <c r="F109" s="13" t="n">
@@ -23145,7 +23145,7 @@
         <v>322</v>
       </c>
       <c r="D116" s="13" t="s">
-        <v>323</v>
+        <v>1062</v>
       </c>
       <c r="E116" s="13"/>
       <c r="F116" s="13" t="n">
@@ -23251,7 +23251,7 @@
         <v>322</v>
       </c>
       <c r="D121" s="13" t="s">
-        <v>323</v>
+        <v>1062</v>
       </c>
       <c r="E121" s="13"/>
       <c r="F121" s="13" t="n">
@@ -23321,7 +23321,7 @@
         <v>322</v>
       </c>
       <c r="D124" s="13" t="s">
-        <v>323</v>
+        <v>1062</v>
       </c>
       <c r="E124" s="13"/>
       <c r="F124" s="13" t="n">
@@ -23363,7 +23363,7 @@
         <v>322</v>
       </c>
       <c r="D126" s="13" t="s">
-        <v>323</v>
+        <v>1062</v>
       </c>
       <c r="E126" s="13"/>
       <c r="F126" s="13" t="n">
@@ -23429,7 +23429,7 @@
         <v>322</v>
       </c>
       <c r="D129" s="13" t="s">
-        <v>323</v>
+        <v>1062</v>
       </c>
       <c r="E129" s="13"/>
       <c r="F129" s="13" t="n">
@@ -23497,7 +23497,7 @@
         <v>322</v>
       </c>
       <c r="D132" s="13" t="s">
-        <v>323</v>
+        <v>1062</v>
       </c>
       <c r="E132" s="13"/>
       <c r="F132" s="13" t="n">
@@ -23539,7 +23539,7 @@
         <v>322</v>
       </c>
       <c r="D134" s="13" t="s">
-        <v>323</v>
+        <v>1062</v>
       </c>
       <c r="E134" s="13"/>
       <c r="F134" s="13" t="n">
@@ -23585,7 +23585,7 @@
         <v>322</v>
       </c>
       <c r="D136" s="13" t="s">
-        <v>323</v>
+        <v>1062</v>
       </c>
       <c r="E136" s="13"/>
       <c r="F136" s="13" t="n">
@@ -23627,7 +23627,7 @@
         <v>322</v>
       </c>
       <c r="D138" s="13" t="s">
-        <v>323</v>
+        <v>1062</v>
       </c>
       <c r="E138" s="13"/>
       <c r="F138" s="13" t="n">
@@ -24283,7 +24283,7 @@
         <v>322</v>
       </c>
       <c r="D170" s="13" t="s">
-        <v>323</v>
+        <v>1062</v>
       </c>
       <c r="E170" s="13"/>
       <c r="F170" s="13" t="n">
@@ -24431,7 +24431,7 @@
         <v>322</v>
       </c>
       <c r="D177" s="13" t="s">
-        <v>323</v>
+        <v>1062</v>
       </c>
       <c r="E177" s="13"/>
       <c r="F177" s="13" t="n">

</xml_diff>